<commit_message>
Verification plan rev2: scope-pure content, human wording, architecture-aligned names
- Strip every guideline/team reference — sheets read as the team's own
  engineering requirements
- Delete all checks/probes for out-of-goal features (irq ack, debug status,
  core_sleep, mep c/mcause sideband probe) — static tie-off driving only
- Narrow illegal-encoding stimulus to RV32I/M space (a/b/c categories);
  F/A/custom/CSR opcodes simply never generated
- Rename all components/monitors to match the UVM architecture diagram
  (if_agent, if_passive_agent, lsu_agent, lsu_passive_agent, rvfi_monitor,
  uvm_scoreboard, ref_model, sva_module, sys_ctrl_agent)
- 55 System / 42 Generation / 45 Checking / 40 Coverage / 27 tests

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/verification plan final/risc_v_verification_plan.xlsx
+++ b/verification plan final/risc_v_verification_plan.xlsx
@@ -472,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D61"/>
+  <dimension ref="A1:D57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20.7" customWidth="1" min="1" max="1"/>
@@ -516,12 +516,12 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>DUT is cv32e40p_top with default parameters (COREV_PULP=0, COREV_CLUSTER=0, FPU=0, FPU_ADDMUL_LAT=0, FPU_OTHERS_LAT=0, ZFINX=0, NUM_MHPMCOUNTERS=1). Effective ISA: RV32I + M + (C, Zicsr, Zicntr, Zifencei out of verification scope). mimpid = 0.</t>
+          <t>DUT is cv32e40p_top with default parameters (COREV_PULP=0, COREV_CLUSTER=0, FPU=0, FPU_ADDMUL_LAT=0, FPU_OTHERS_LAT=0, ZFINX=0, NUM_MHPMCOUNTERS=1). Effective ISA: RV32I + M (the C, Zicsr, Zicntr and Zifencei extensions exist in hardware but are outside the verification goal). mimpid = 0.</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>Instantiate rtl/cv32e40p_top.sv (core; no FPU wrapper inside because FPU=0). Verification is top-level (core as a whole) per guideline Team2 Q2.</t>
+          <t>top_tb instantiates rtl/cv32e40p_top.sv and verifies the core as a whole at top level.</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
@@ -543,12 +543,12 @@
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>One UVM interface per agent group: sys_ctrl_if, if_obi_if, lsu_obi_if, rvfi internal probes.</t>
+          <t>Four virtual interfaces wrap the pins: sys_ctrl_vif, if_vif, lsu_vif and rvfi_vif (internal probes).</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>top_tb, sys_ctrl_agent, if_agt, lsu_agt, rvfi_pas_mon</t>
+          <t>top_tb, sys_ctrl_agent, if_agent, lsu_agent, rvfi_monitor</t>
         </is>
       </c>
     </row>
@@ -570,7 +570,7 @@
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>sys_ctrl_agent, if_pas_mon, lsu_pas_mon</t>
+          <t>sys_ctrl_agent, if_passive_agent, lsu_passive_agent</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
       <c r="C6" s="5" t="inlineStr"/>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>sys_ctrl_agent, if_pas_mon</t>
+          <t>sys_ctrl_agent, if_passive_agent</t>
         </is>
       </c>
     </row>
@@ -605,12 +605,12 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Exceptions always to base, verified via rtl cv32e40p_if_stage.sv EXC_PC_EXCEPTION mux.</t>
+          <t>Exceptions always go to the base, as implemented in cv32e40p_if_stage.sv (EXC_PC_EXCEPTION mux).</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>sys_ctrl_agent, if_pas_mon, sb</t>
+          <t>sys_ctrl_agent, if_passive_agent, uvm_scoreboard</t>
         </is>
       </c>
     </row>
@@ -622,17 +622,17 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>fetch_enable_i: the first instruction fetch after reset de-assertion must not happen while fetch_enable_i==0; after fetch_enable_i has been 1 for at least one cycle (out of reset) fetching starts permanently, and the value of fetch_enable_i is ignored until the next reset. boot_addr_i/mtvec_addr_i/dm_*_addr_i/hart_id_i must stay stable once enabled.</t>
+          <t>fetch_enable_i: the first instruction fetch after reset de-assertion must not happen while fetch_enable_i==0; after fetch_enable_i has been 1 for at least one cycle (out of reset) fetching starts permanently, and the value of fetch_enable_i is ignored until the next reset. boot_addr_i / mtvec_addr_i / dm_*_addr_i / hart_id_i must stay stable once the core is enabled.</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Internal clock is gated until fetch_enable_i (sleep unit).</t>
+          <t>The internal clock is gated until fetch_enable_i (sleep unit).</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>sys_ctrl_agent, if_pas_mon</t>
+          <t>sys_ctrl_agent, if_passive_agent</t>
         </is>
       </c>
     </row>
@@ -644,13 +644,17 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Out-of-scope input pins are tied off for the whole simulation: irq_i = 32'b0, debug_req_i = 1'b0, pulp_clock_en_i = 1'b0, scan_cg_en_i = 1'b0 (guideline Team1 Q3: minimal work so out-of-scope logic never hinders the main task).</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr"/>
+          <t>To keep the core in normal operation, the inputs that belong to out-of-goal features are driven to static values for the entire simulation: irq_i = 32'b0, debug_req_i = 1'b0, pulp_clock_en_i = 1'b0, scan_cg_en_i = 1'b0.</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Static driving only; no checkers or coverage are built for these features.</t>
+        </is>
+      </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>sys_ctrl_agent</t>
+          <t>sys_ctrl_agent (driver)</t>
         </is>
       </c>
     </row>
@@ -662,339 +666,281 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>With irq_i tied to 0, no interrupt may ever be taken: irq_ack_o must stay 0 for the whole simulation.</t>
+          <t>Primary outputs of cv32e40p_top must never be X/Z after reset de-assertion while the core is clocked: instr_req_o, instr_addr_o, data_req_o, data_we_o, data_be_o, data_addr_o, data_wdata_o (when driven).</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr"/>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>sys_ctrl_agent, rvfi_pas_mon</t>
+          <t>if_passive_agent, lsu_passive_agent</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>risc_sys_08</t>
+          <t>risc_if_00</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>With debug_req_i tied to 0 and no ebreak stimulus, the core must never enter Debug Mode: debug_halted_o must stay 0 after startup. debug_havereset_o / debug_running_o / debug_halted_o are mutually exclusive (exactly one asserted at any time); debug_havereset_o is set during reset and clears a few cycles after reset de-assert with fetch_enable_i high.</t>
+          <t>Instruction fetch OBI handshake: instr_req_o is raised for a fetch and must stay high until instr_gnt_i is sampled high for one cycle (request persistence - a request must never be retracted or its address changed once issued).</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Debug interface behavior per databook debug chapter; debug module itself out of scope.</t>
+          <t>The address phase ends at the gnt cycle; instr_addr_o may change the cycle after.</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>sys_ctrl_agent, rvfi_pas_mon</t>
+          <t>if_agent, if_passive_agent</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>risc_sys_09</t>
+          <t>risc_if_01</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>core_sleep_o must stay 0 for the whole simulation: no wfi and no cv.elw are ever generated (out of scope), so the internal clock is never gated after fetch_enable_i.</t>
+          <t>instr_req_o must not combinationally depend on instr_rvalid_i (OBI: no rvalid-&gt;req dependency); instr_gnt_i may be high even when there is no request, which must not cause any spurious side effect.</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr"/>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>sys_ctrl_agent</t>
+          <t>if_agent, if_passive_agent</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>risc_sys_10</t>
+          <t>risc_if_02</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Primary outputs of cv32e40p_top must never be X/Z after reset de-assertion while the core is clocked: instr_req_o, instr_addr_o, data_req_o, data_we_o, data_be_o, data_addr_o, data_wdata_o (when driven).</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr"/>
+          <t>Response phase: instr_rvalid_i is high for exactly one cycle per granted request; instr_rdata_i is sampled in that cycle. Responses must arrive in issue order (master point of view), possibly one or more cycles after grant; the IF interface can have up to DEPTH=2 outstanding requests.</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>The TB memory enforces in-order responses; the core relies on ordering (no IDs).</t>
+        </is>
+      </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>if_pas_mon, lsu_pas_mon</t>
+          <t>if_agent, if_passive_agent</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>risc_if_00</t>
+          <t>risc_if_03</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Instruction fetch OBI handshake: instr_req_o is raised for a fetch and must stay high until instr_gnt_i is sampled high for one cycle (request persistence - a request must never be retracted or its address changed once issued).</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>Address phase ends at the gnt cycle; instr_addr_o may change the cycle after.</t>
-        </is>
-      </c>
+          <t>Back-to-back fetches: while the prefetch FIFO drains, a new instr_req_o may be issued in the cycle immediately following a gnt; a continuous request stream must be sustained.</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr"/>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>if_agt, if_pas_mon</t>
+          <t>if_agent, if_passive_agent</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>risc_if_01</t>
+          <t>risc_if_04</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>instr_req_o must not combinationally depend on instr_rvalid_i (OBI: no rvalid-&gt;req dependency); instr_gnt_i may be high even when there is no request, which must not cause any spurious side effect.</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr"/>
+          <t>Speculative prefetch: the core may fetch up to DEPTH=2 32-bit words beyond the currently executed code region; the instruction memory model must serve any address without side effects and must tolerate reads past the program end.</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Direct consequence of the prefetch buffer; the TB memory never assumes fetch==execute.</t>
+        </is>
+      </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>if_agt, if_pas_mon</t>
+          <t>if_agent (instr_mem_model)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>risc_if_02</t>
+          <t>risc_if_05</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Response phase: instr_rvalid_i is high for exactly one cycle per granted request; instr_rdata_i is sampled in that cycle. Responses must arrive in issue order (master point of view), possibly one or more cycles after grant; the IF interface can have up to DEPTH=2 outstanding requests.</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>TB memory enforces in-order; core relies on ordering (no IDs).</t>
-        </is>
-      </c>
+          <t>Flush on taken jump (JAL/JALR are resolved in the ID stage): the prefetch buffer and IF stage are flushed; the new PC request appears on the instruction-side memory interface in the same cycle the jump is in ID; with zero wait states the jump costs 2 cycles.</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr"/>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>if_agt, if_pas_mon</t>
+          <t>if_passive_agent, uvm_scoreboard</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>risc_if_03</t>
+          <t>risc_if_06</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>Back-to-back fetches: while the prefetch FIFO drains, a new instr_req_o may be issued in the cycle immediately following a gnt; a continuous request stream must be sustained.</t>
+          <t>Flush on taken branch (resolved in the EX stage): the IF stage and ID stage are flushed; fetch restarts at the branch target; with zero wait states a taken branch costs 3 cycles; a not-taken branch costs 1 cycle (no stall).</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr"/>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>if_agt, if_pas_mon</t>
+          <t>if_passive_agent, uvm_scoreboard</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>risc_if_04</t>
+          <t>risc_if_07</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Speculative prefetch: the core may fetch up to DEPTH=2 32-bit words beyond the currently executed code region; the instruction memory model must serve any address without side effects and must tolerate reads past the program end.</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
-          <t>Direct consequence of prefetch buffer; TB memory must never assume fetch==execute.</t>
-        </is>
-      </c>
+          <t>Flush on trap (illegal instruction): the pipeline is flushed and fetch restarts at the mtvec base address; handler code at the base continues normally afterwards.</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr"/>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>if_agt (instr_mem_model)</t>
+          <t>if_passive_agent, uvm_scoreboard</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>risc_if_05</t>
+          <t>risc_if_08</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>Flush on taken jump (JAL/JALR are resolved in ID stage): the prefetch buffer and IF stage are flushed; the new PC request appears on the instruction-side memory interface in the same cycle the jump is in ID; with zero wait states the jump costs 2 cycles.</t>
-        </is>
-      </c>
-      <c r="C19" s="5" t="inlineStr"/>
+          <t>Stimulus constraint: all generated programs consist of 32-bit instructions only, word-aligned (no RVC encodings), with word-aligned branch/jump targets; programs are bounded and terminate at a defined end-of-program sentinel address recognized by the teardown. The aligner and compressed decoder belong to the never-tested C extension and are exercised only as pass-through hardware.</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>No self-modifying code is generated (it would require fence.i, which is omitted from the stimulus).</t>
+        </is>
+      </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>if_pas_mon, sb</t>
+          <t>generation constraint (riscv_program)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>risc_if_06</t>
+          <t>risc_if_09</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>Flush on taken branch (resolved in EX stage): IF stage and ID stage are flushed; fetch restarts at the branch target; with zero wait states a taken branch costs 3 cycles; a not-taken branch costs 1 cycle (no stall).</t>
-        </is>
-      </c>
-      <c r="C20" s="5" t="inlineStr"/>
+          <t>No instruction-address-misaligned exception exists in this core (the C extension is always enabled), so instruction fetch must never cause a trap; any trap observed on a legal stream is a bug.</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Sanity/anti-check.</t>
+        </is>
+      </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>if_pas_mon, sb</t>
+          <t>uvm_scoreboard</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>risc_if_07</t>
+          <t>risc_lsu_00</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>Flush on trap (illegal instruction): the pipeline is flushed and fetch restarts at the mtvec base address; handler code at the base continues normally afterwards.</t>
+          <t>Data OBI handshake: data_req_o is raised for load/store and must stay high until data_gnt_i is sampled high; data_addr_o, data_we_o, data_be_o, data_wdata_o are sent together with the request and must stay stable while req==1 &amp;&amp; gnt==0.</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr"/>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>if_pas_mon, sb</t>
+          <t>lsu_agent, lsu_passive_agent</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>risc_if_08</t>
+          <t>risc_lsu_01</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>Stimulus constraint: all generated programs consist of 32-bit instructions only, word-aligned (no RVC encodings), with word-aligned branch/jump targets; programs are bounded and terminate at a defined end-of-program sentinel address recognized by the teardown. The aligner and compressed decoder are part of the never-tested C extension per guideline Team2 Q1 and are exercised only as pass-through hardware.</t>
-        </is>
-      </c>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t>No self-modifying code is generated (would require fence.i, which is excluded per guideline Team4 Q2).</t>
-        </is>
-      </c>
+          <t>Response phase (data side): data_rvalid_i is high for exactly one cycle per granted request and terminates both read and write transactions (for stores data_rdata_i is meaningless). Responses are in issue order; the data interface supports up to 2 outstanding transactions; when responses lag, the core applies back-pressure (EX/WB stall) instead of issuing further requests.</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr"/>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>generation constraint (riscv_program)</t>
+          <t>lsu_agent, lsu_passive_agent</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>risc_if_09</t>
+          <t>risc_lsu_02</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>No instruction-address-misaligned exception exists in this core (the C extension is always enabled), so instruction fetch must never cause a trap; any trap observed on a legal stream is a bug.</t>
+          <t>With zero wait states, Load/Store is handled in 1 bus transaction using both EX and WB stages for 1 cycle each (databook cycle table); a non-word-aligned word transfer, or a halfword transfer crossing a word boundary, takes 2 bus transactions (see risc_lsu_04); a store completes when its rvalid returns. cv.elw is out of scope.</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>Sanity/anti-check.</t>
+          <t>Informational timing, verified through latency coverage at zero-wait.</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>sb</t>
+          <t>lsu_passive_agent, uvm_scoreboard</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>risc_lsu_00</t>
+          <t>risc_lsu_03</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
-        <is>
-          <t>Data OBI handshake: data_req_o is raised for load/store and must stay high until data_gnt_i is sampled high; data_addr_o, data_we_o, data_be_o, data_wdata_o are send together with the request and must stay stable while req==1 &amp;&amp; gnt==0.</t>
-        </is>
-      </c>
-      <c r="C24" s="5" t="inlineStr"/>
-      <c r="D24" s="5" t="inlineStr">
-        <is>
-          <t>lsu_agt, lsu_pas_mon</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="5" t="inlineStr">
-        <is>
-          <t>risc_lsu_01</t>
-        </is>
-      </c>
-      <c r="B25" s="5" t="inlineStr">
-        <is>
-          <t>Response phase (data side): data_rvalid_i is high for exactly one cycle per granted request and terminates both read and write transactions (for stores data_rdata_i is meaningless). Responses are in issue order; the data interface supports up to 2 outstanding transactions; when responses lag, the core applies back-pressure (EX/WB stall) instead of issuing further requests.</t>
-        </is>
-      </c>
-      <c r="C25" s="5" t="inlineStr"/>
-      <c r="D25" s="5" t="inlineStr">
-        <is>
-          <t>lsu_agt, lsu_pas_mon</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="5" t="inlineStr">
-        <is>
-          <t>risc_lsu_02</t>
-        </is>
-      </c>
-      <c r="B26" s="5" t="inlineStr">
-        <is>
-          <t>With zero wait states, Load/Store is handled in 1 bus transaction using both EX and WB stages for 1 cycle each (databook cycle table); a non-word-aligned word transfer, or a halfword transfer crossing a word boundary, takes 2 bus transactions (see risc_lsu_04); a store completes when its rvalid returns. cv.elw is out of scope.</t>
-        </is>
-      </c>
-      <c r="C26" s="5" t="inlineStr">
-        <is>
-          <t>Informational timing, verified through latency coverage at zero-wait.</t>
-        </is>
-      </c>
-      <c r="D26" s="5" t="inlineStr">
-        <is>
-          <t>lsu_pas_mon, sb</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="5" t="inlineStr">
-        <is>
-          <t>risc_lsu_03</t>
-        </is>
-      </c>
-      <c r="B27" s="5" t="inlineStr">
         <is>
           <t>Byte-enable generation per access type and address (from rtl cv32e40p_load_store_unit.sv):
 SW: addr[1:0]=00-&gt;4'b1111; misaligned first beat 01-&gt;1110, 10-&gt;1100, 11-&gt;1000; second beat 01-&gt;0001, 10-&gt;0011, 11-&gt;0111.
@@ -1003,676 +949,657 @@
 Only these patterns may ever appear on data_be_o.</t>
         </is>
       </c>
+      <c r="C24" s="5" t="inlineStr"/>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>lsu_passive_agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>risc_lsu_04</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>Misaligned handling: the LSU never raises address-misaligned exceptions. A word load/store at addr[1:0]!=00, or a halfword at addr[1:0]==11, is performed as TWO bus transactions; the transfer for the lowest address is issued first, followed by (aligned base+4) with the complementary byte-enables; the memory transfers for the two parts are merged by the core into one load/store view. All other offsets need a single transaction.</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>Verified in rtl cv32e40p_load_store_unit.sv (data_misaligned_o, misaligned_st) and the databook LSU chapter.</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>lsu_passive_agent, uvm_scoreboard</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>risc_lsu_05</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Store data alignment: data_wdata_o is rotated by wdata_offset = addr[1:0] - reg_offset[1:0] (rtl formula), i.e. 01-&gt;{wdata[23:0],wdata[31:24]}, 10-&gt;{wdata[15:0],wdata[31:16]}, 11-&gt;{wdata[7:0],wdata[31:8]}; the memory applies data_be_o lanes only.</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr"/>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>lsu_passive_agent, uvm_scoreboard</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>risc_lsu_06</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Load data alignment and extension: LB/LH sign-extend the addressed byte/halfword; LBU/LHU zero-extend; LW returns the full word; for misaligned accesses the two response words are assembled (first-response low bytes kept in rdata_q, combined with the second response) according to the address offset.</t>
+        </is>
+      </c>
       <c r="C27" s="5" t="inlineStr"/>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>lsu_pas_mon</t>
+          <t>uvm_scoreboard</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>risc_lsu_04</t>
+          <t>risc_lsu_07</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>Misaligned handling: the LSU never raises address-misaligned exceptions. A word load/store at addr[1:0]!=00, or a halfword at addr[1:0]==11, is performed as TWO bus transactions; the transfer for the lowest address is issued first, followed by (aligned base+4) with the complementary byte-enables; the core spends 2 cycles each in EX and WB per part and merges the response data. All other offsets need a single transaction.</t>
+          <t>Memory consistency: in-order data responses and a single hart imply a load must observe the value of the most recent previously-issued store to the same byte address; the TB memory model commits a store at its rvalid and never reorders.</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>Databook LSU chapter + verified in rtl (data_misaligned_o / misaligned_st logic).</t>
+          <t>No store buffer exists in the core; the end-to-end behavior is still checked explicitly.</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>lsu_pas_mon, sb</t>
+          <t>uvm_scoreboard</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>risc_lsu_05</t>
+          <t>risc_lsu_08</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>Store data alignment: data_wdata_o is rotated by wdata_offset = addr[1:0] - reg_offset[1:0] (rtl formula), i.e. 01-&gt;{wdata[23:0],wdata[31:24]}, 10-&gt;{wdata[15:0],wdata[31:16]}, 11-&gt;{wdata[7:0],wdata[31:8]}; the memory applies data_be_o lanes only.</t>
+          <t>Flushed instructions must not affect the data bus: loads/stores younger than a taken branch, jump, or trap (still in IF/ID) are killed before their request phase - no spurious data_req_o from flushed instructions may appear.</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr"/>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>lsu_pas_mon, sb</t>
+          <t>lsu_passive_agent, uvm_scoreboard</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>risc_lsu_06</t>
+          <t>risc_lsu_09</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>Load data alignment and extension: LB/LH sign-extend the addressed byte/halfword; LBU/LHU zero-extend; LW returns the full word; for misaligned accesses the two response words are assembled (first-response low bytes kept in rdata_q, combined with second response) according to the address offset.</t>
-        </is>
-      </c>
-      <c r="C30" s="5" t="inlineStr"/>
+          <t>The data OBI interface has no error response signal; the TB memory always completes transactions successfully - no error stimulus is generated or expected.</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>The load_err/store_err paths in the RTL are tied inactive in this configuration (no PMP).</t>
+        </is>
+      </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>sb</t>
+          <t>lsu_agent</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>risc_lsu_07</t>
+          <t>risc_dec_00</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>Memory consistency: in-order data responses + single hart imply a load must observe the value of the most recent previously-issued store to the same byte address; the TB memory model commits a store at its rvalid and never reorders.</t>
+          <t>All RV32I base instructions are legal and must execute correctly: LUI, AUIPC, JAL, JALR, BEQ, BNE, BLT, BGE, BLTU, BGEU, LB, LH, LW, LBU, LHU, SB, SH, SW, ADDI, SLTI, SLTIU, XORI, ORI, ANDI, SLLI, SRLI, SRAI, ADD, SUB, SLL, SLT, SLTU, XOR, SRL, SRA, OR, AND. (FENCE / FENCE.I / ECALL / EBREAK are part of the base ISA but are omitted from the generated stimulus.)</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>No store buffer in the core; ordering is trivially program order, but must be checked end-to-end.</t>
+          <t>Golden reference: an in-house RV32IM model connected to the uvm_scoreboard.</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>sb</t>
+          <t>uvm_scoreboard, ref_model</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>risc_lsu_08</t>
+          <t>risc_dec_01</t>
         </is>
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>Flushed instructions must not affect the data bus: loads/stores younger than a taken branch, jump, or trap (still in IF/ID) are killed before their request phase - no spurious data_req_o from flushed instructions may appear.</t>
+          <t>All 8 RV32M instructions are legal and must execute correctly: MUL, MULH, MULHSU, MULHU, DIV, DIVU, REM, REMU.</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr"/>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>lsu_pas_mon, sb</t>
+          <t>uvm_scoreboard, ref_model</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>risc_lsu_09</t>
+          <t>risc_dec_02</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>The data OBI interface has no error response (no err signal); the TB memory always completes transactions successfully - no error stimulus is generated or expected.</t>
+          <t>Illegal instruction detection within the RV32I/M opcode space (verified against cv32e40p_decoder.sv illegal_insn conditions): any undefined encoding raises an illegal instruction exception, including:
+(a) undefined major opcodes;
+(b) a legal major opcode with an undefined funct3/funct7 combination;
+(c) reserved shift encodings: OP-IMM/OP with funct3=001/101 and imm[11:5] (funct7) other than 0000000 or 0100000.</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>load_err_o/store_err_o paths in rtl are tied inactive (no PMP in this config).</t>
+          <t>Encodings of disabled extensions (FPU/atomic/CORE-V custom/CSR opcodes) are never generated at all - see risc_dec_04.</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>lsu_agt</t>
+          <t>uvm_scoreboard, if_passive_agent</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>risc_dec_00</t>
+          <t>risc_dec_03</t>
         </is>
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>All RV32I base instructions are legal and must execute correctly: LUI, AUIPC, JAL, JALR, BEQ, BNE, BLT, BGE, BLTU, BGEU, LB, LH, LW, LBU, LHU, SB, SH, SW, ADDI, SLTI, SLTIU, XORI, ORI, ANDI, SLLI, SRLI, SRAI, ADD, SUB, SLL, SLT, SLTU, XOR, SRL, SRA, OR, AND. (FENCE/FENCE.I/ECALL/EBREAK are part of the base but are excluded from stimulus per guideline Team4 Q2.)</t>
-        </is>
-      </c>
-      <c r="C34" s="5" t="inlineStr">
-        <is>
-          <t>Golden reference = in-house RV32IM model inside the scoreboard (guideline Team2 Q7: build everything yourself).</t>
-        </is>
-      </c>
+          <t>Register operands equal to x0 keep legality: e.g. ADD x0,rs1,rs2, loads with rd=x0, JAL x0 (no link) are legal and produce the standard no-write/no-link behavior (see risc_rf_00); encodings that are undefined remain illegal even with x0 fields.</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr"/>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>sb, ref_model</t>
+          <t>uvm_scoreboard</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>risc_dec_01</t>
+          <t>risc_dec_04</t>
         </is>
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>All 8 RV32M instructions are legal and must execute correctly: MUL, MULH, MULHSU, MULHU, DIV, DIVU, REM, REMU.</t>
-        </is>
-      </c>
-      <c r="C35" s="5" t="inlineStr"/>
+          <t>Omitted from stimulus (generation constraint): FENCE, FENCE.I, ECALL, EBREAK, WFI, MRET and all CSR instructions; interrupt and debug traffic; compressed instructions; all FPU / CORE-V custom / atomic instructions (including their opcodes as partial encodings).</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>Generation constraint only - no checkers or coverage are built for these.</t>
+        </is>
+      </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>sb, ref_model</t>
+          <t>generation constraint (riscv_program)</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>risc_dec_02</t>
+          <t>risc_alu_00</t>
         </is>
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>Illegal instruction detection (verified against cv32e40p_decoder.sv illegal_insn conditions): any encoding undefined for the configured parameter set raises an illegal instruction exception, including:
-(a) undefined major opcodes;
-(b) legal major opcode with undefined funct3/funct7 combination;
-(c) reserved shift encodings: OP-IMM/OP with funct3=001/101 and imm[11:5] (funct7) other than 0000000 or 0100000;
-(d) F / D / A major opcodes (FPU=0, atomics removed); (e) SYSTEM/CSR instructions accessing unimplemented CSR addresses; (f) CORE-V custom opcode spaces (incl. 0x0B, 0x2B, 0x5B, 0x7B) while COREV_PULP=0 / COREV_CLUSTER=0.</t>
-        </is>
-      </c>
-      <c r="C36" s="5" t="inlineStr">
-        <is>
-          <t>Guideline Team2 Q10 confirms reserved-shift encodings are in the illegal scope.</t>
-        </is>
-      </c>
+          <t>Integer computational instructions (ADD/SUB/AND/OR/XOR/SLL/SRL/SRA/SLT/SLTU + I-forms, LUI, AUIPC) produce their result in 1 cycle; the EX-&gt;ID forwarding path gives a 0-cycle penalty for a back-to-back dependent ALU instruction; SLT/SLTU distinguish signed vs unsigned compare and SLTIU compares rs1 unsigned against the sign-extended immediate (per the RISC-V spec).</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr"/>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>sb, if_pas_mon</t>
+          <t>uvm_scoreboard</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
         <is>
-          <t>risc_dec_03</t>
+          <t>risc_alu_01</t>
         </is>
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>Trap state update on illegal instruction: mepc &lt;- PC of the offending instruction, mcause &lt;- 2 (illegal instruction), mstatus.MPIE/MIE update; PC &lt;- mtvec base. CSR content verification itself is out of scope; the architecturally visible effect (fetch redirect, no side effects) is checked, and mepc/mcause are probed only optionally.</t>
-        </is>
-      </c>
-      <c r="C37" s="5" t="inlineStr">
-        <is>
-          <t>Scoreboard checks redirect; optional hierarchical probe on mepc/mcause kept as commented-out check.</t>
-        </is>
-      </c>
+          <t>Shifts use a single-cycle barrel shifter; the shift amount shamt is operand_b[4:0] (register form) or imm[4:0]; SRA/SRAI replicate the sign bit; SLL/SRL shift in zeros. shamt=0 leaves the operand unchanged.</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr"/>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>sb</t>
+          <t>uvm_scoreboard</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
         <is>
-          <t>risc_dec_04</t>
+          <t>risc_alu_02</t>
         </is>
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>Register operands equal to x0 keep legality: e.g. ADD x0,rs1,rs2, loads with rd=x0, JAL x0 (no link) are legal and produce the standard no-write/no-link behavior (see risc_rf_00); encodings that are undefined remain illegal even with x0 fields.</t>
+          <t>LUI writes imm[31:12]&lt;&lt;12; AUIPC writes PC + (imm&lt;&lt;12) - the result depends on the current PC (position-dependent behavior).</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr"/>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>sb</t>
+          <t>uvm_scoreboard</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
         <is>
-          <t>risc_dec_05</t>
+          <t>risc_m_00</t>
         </is>
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>Excluded from stimulus per guidelines (Team2 Q5, Team3, Team4 Q2/Q3, Team5 Q3): FENCE, FENCE.I, ECALL, EBREAK, WFI, MRET and all CSR instructions; interrupt and debug traffic; compressed instructions; all FPU/PULP/atomic instructions (they only appear as illegal-encoding injections, never as legal flow).</t>
-        </is>
-      </c>
-      <c r="C39" s="5" t="inlineStr">
-        <is>
-          <t>Out-of-scope row (mirrors template 'Features Not Supported').</t>
-        </is>
-      </c>
+          <t>MUL executes in 1 cycle (32x32 single-cycle multiplier, lower 32 bits of the product).</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr"/>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>generation constraint (riscv_program)</t>
+          <t>uvm_scoreboard</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
-          <t>risc_alu_00</t>
+          <t>risc_m_01</t>
         </is>
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>Integer computational instructions (ADD/SUB/AND/OR/XOR/SLL/SRL/SRA/SLT/SLTU + I-forms, LUI, AUIPC) produce their result in 1 cycle; the EX-&gt;ID forwarding path provides a 0-cycle penalty for a back-to-back dependent ALU instruction; SLT/SLTU distinguish signed vs unsigned compare and SLTIU compares rs1 unsigned against the sign-extended immediate (per RISC-V spec).</t>
+          <t>MULH/MULHSU/MULHU take 5 cycles (multicycle FSM STEP0-&gt;STEP1-&gt;STEP2-&gt;FINISH in rtl cv32e40p_mult.sv) and stall EX meanwhile; they return the upper 32 bits for signed x signed, signed x unsigned, unsigned x unsigned operands respectively.</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr"/>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>sb</t>
+          <t>uvm_scoreboard</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t>risc_alu_01</t>
+          <t>risc_m_02</t>
         </is>
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>Shifts use a single-cycle barrel shifter; shift amount shamt is operand_b[4:0] (reg form) or imm[4:0]; SRA/SRAI replicate the sign bit; SLL/SRL shift in zeros. shamt=0 leaves the operand unchanged.</t>
-        </is>
-      </c>
-      <c r="C41" s="5" t="inlineStr"/>
+          <t>DIV/DIVU/REM/REMU are iterative with early termination: latency is 3..35 cycles depending on the number of leading zeros of operand b (the divisor); minimum 3 cycles when the divisor has no leading zeros (e.g. 0x80000000), maximum 35 when the divisor is 0; EX stalls meanwhile.</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>Early-termination loop verified in rtl cv32e40p_alu_div.sv (the divisor is pre-shifted).</t>
+        </is>
+      </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>sb</t>
+          <t>uvm_scoreboard, lsu_passive_agent</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
         <is>
-          <t>risc_alu_02</t>
+          <t>risc_m_03</t>
         </is>
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>LUI writes imm[31:12]&lt;&lt;12; AUIPC writes PC + (imm&lt;&lt;12) - the value depends on the current PC (position-dependent behavior).</t>
+          <t>Special division results per the RISC-V spec: divide-by-zero -&gt; quotient = -1 (all ones) for DIV/DIVU; remainder = dividend for REM/REMU. Signed overflow (DIV -2^31 / -1) -&gt; quotient = -2^31, REM -2^31 / -1 -&gt; 0. The REM sign follows the dividend; REMU is unsigned.</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr"/>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>sb</t>
+          <t>uvm_scoreboard</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
         <is>
-          <t>risc_m_00</t>
+          <t>risc_m_04</t>
         </is>
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>MUL executes in 1 cycle (32x32 single-cycle multiplier, lower 32 bits of the product).</t>
-        </is>
-      </c>
-      <c r="C43" s="5" t="inlineStr"/>
+          <t>A multicycle instruction (MULH/DIV/REM) that is older than a taken branch always completes and writes back normally, even when the flush of the younger path lands in the same window - only IF/ID (the younger stages) are flushed.</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>Consistent with the databook pipeline chapter and the controller FSM.</t>
+        </is>
+      </c>
       <c r="D43" s="5" t="inlineStr">
         <is>
-          <t>sb</t>
+          <t>uvm_scoreboard</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="5" t="inlineStr">
         <is>
-          <t>risc_m_01</t>
+          <t>risc_haz_00</t>
         </is>
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>MULH/MULHSU/MULHU take 5 cycles (multicycle FSM STEP0-&gt;STEP1-&gt;STEP2-&gt;FINISH in rtl cv32e40p_mult.sv) and stall EX meanwhile; they return the upper 32 bits for signed x signed, signed x unsigned, unsigned x unsigned operands respectively.</t>
-        </is>
-      </c>
-      <c r="C44" s="5" t="inlineStr"/>
+          <t>RAW forwarding: ALU/MUL/DIV results in EX are forwarded to ID-stage operands (ports a and b), giving a 0-cycle penalty for back-to-back dependent instructions; the consumer reads correct producer values at distance 1, 2, 3.</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>Forwarding muxes verified in rtl cv32e40p_id_stage.sv (reg_d_ex/alu_is_reg_a/b/c).</t>
+        </is>
+      </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>sb</t>
+          <t>uvm_scoreboard</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
         <is>
-          <t>risc_m_02</t>
+          <t>risc_haz_01</t>
         </is>
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>DIV/DIVU/REM/REMU are iterative with early termination: latency is 3..35 cycles depending on the number of leading zeros of operand b (divisor); minimum 3 cycles when the divisor has no leading zeros (e.g. 0x80000000), maximum 35 when the divisor is 0; EX stalls meanwhile.</t>
+          <t>Load-use hazard: an instruction consuming a register written by the immediately preceding load is stalled exactly 1 cycle (controller load_stall + deassert_we in rtl cv32e40p_controller.sv); no wrong value is read and no spurious write occurs during the stall.</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>Latency formula per databook cycle table; early-termination loop verified in rtl/cv32e40p_alu_div.sv (OpBShift pre-shifts divisor).</t>
+          <t>At 1-cycle distance only; &gt;=2-distance consumers are not stalled.</t>
         </is>
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>sb, lsu_pas_mon</t>
+          <t>uvm_scoreboard, rvfi_monitor</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="5" t="inlineStr">
         <is>
-          <t>risc_m_03</t>
+          <t>risc_haz_02</t>
         </is>
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>Special division results per RISC-V spec: Divide-by-zero -&gt; quotient = -1 (all ones) for DIV/DIVU; remainder = dividend for REM/REMU. Signed overflow (DIV -2^31 / -1) -&gt; quotient = -2^31, REM -2^31 / -1 -&gt; 0. REM sign follows the dividend; REMU is unsigned.</t>
+          <t>JALR data hazard: a JALR whose rs1 is produced by the immediately preceding instruction is stalled 1 cycle (jr_stall) before computing its target; the target must be (rs1+imm) &amp; ~1.</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr"/>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>sb</t>
+          <t>uvm_scoreboard</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t>risc_m_04</t>
+          <t>risc_haz_03</t>
         </is>
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>A multicycle instruction (MULH/DIV/REM) that is older than a taken branch always completes and writes back normally even if the flush of younger instructions happens in the same window (answer to open guideline question Team4 Q4, resolved from databook pipeline chapter and rtl: only IF/ID - i.e. younger instructions - are flushed).</t>
+          <t>WAW write-port arbitration: a load in WB and a younger ALU/MUL/DIV instruction in EX may write the same rd in the same cycle; the register file resolves it with port-b (EX) priority, i.e. the architecturally younger instruction wins (verified in rtl cv32e40p_register_file_ff.sv: the we_b write is checked before we_a).</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr"/>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>sb</t>
+          <t>uvm_scoreboard</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="5" t="inlineStr">
         <is>
-          <t>risc_haz_00</t>
+          <t>risc_haz_04</t>
         </is>
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>RAW forwarding: ALU/MUL/DIV results in EX are forwarded to ID-stage operands (ports a and b), giving 0-cycle penalty for back-to-back dependent instructions; the consumer reads correct producer values at distance 1, 2, 3.</t>
-        </is>
-      </c>
-      <c r="C48" s="5" t="inlineStr">
-        <is>
-          <t>Forwarding muxes verified in rtl/cv32e40p_id_stage.sv (reg_d_ex/alu_is_reg_a/b/c).</t>
-        </is>
-      </c>
+          <t>Control-flush cleanliness: instructions younger than a taken branch / jump / trap never produce architectural side effects (no register write, no memory request).</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr"/>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>sb</t>
+          <t>uvm_scoreboard, lsu_passive_agent</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
         <is>
-          <t>risc_haz_01</t>
+          <t>risc_rf_00</t>
         </is>
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>Load-use hazard: an instruction consuming a register written by the immediately preceding load is stalled exactly 1 cycle (controller load_stall + deassert_we in rtl cv32e40p_controller.sv); no wrong value is read and no spurious write occurs during the stall.</t>
-        </is>
-      </c>
-      <c r="C49" s="5" t="inlineStr">
-        <is>
-          <t>At 1-cycle distance only; &gt;=2-distance consumers are not stalled.</t>
-        </is>
-      </c>
+          <t>x0 is hardwired to zero: reads always return 0 and writes to x0 are ignored (x0 has no flip-flops), even when a load targets x0.</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr"/>
       <c r="D49" s="5" t="inlineStr">
         <is>
-          <t>sb, rvfi_pas_mon</t>
+          <t>uvm_scoreboard, rvfi_monitor</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
         <is>
-          <t>risc_haz_02</t>
+          <t>risc_rf_01</t>
         </is>
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>JALR data hazard: a JALR whose rs1 is produced by the immediately preceding instruction is stalled 1 cycle (jr_stall) before computing its target; the target must be (rs1+imm) &amp; ~1.</t>
-        </is>
-      </c>
-      <c r="C50" s="5" t="inlineStr"/>
+          <t>All 31 general-purpose registers x1..x31 are implemented (the FF register file resets to 0 at rst_ni==0) with 3 read ports and 2 write ports; reads happen in ID, writes from EX and WB.</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>Reset-zero is an implementation property of the FF-based register file - checked once at test start; it is not an ISA requirement.</t>
+        </is>
+      </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
-          <t>sb</t>
+          <t>uvm_scoreboard</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="5" t="inlineStr">
         <is>
-          <t>risc_haz_03</t>
+          <t>risc_rst_00</t>
         </is>
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>WAW write-port arbitration: a load in WB and a younger ALU/MUL/DIV instruction in EX may write the same rd in the same cycle; the register file resolves it with port-b (EX) priority, i.e. the architecturally younger instruction wins (open guideline question Team4 Q6, answered directly from rtl cv32e40p_register_file_ff.sv: we_b checked before we_a).</t>
-        </is>
-      </c>
-      <c r="C51" s="5" t="inlineStr"/>
+          <t>Reset re-assertion during an outstanding instruction-fetch transaction: core and TB slave both drop the transaction; after re-enabling, the core re-boots from boot_addr_i with a clean pipeline; no stale rvalid may be consumed after reset.</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>TB OBI slaves implement a reset that clears their outstanding queues.</t>
+        </is>
+      </c>
       <c r="D51" s="5" t="inlineStr">
         <is>
-          <t>sb</t>
+          <t>sys_ctrl_agent, if_agent, uvm_scoreboard</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="5" t="inlineStr">
         <is>
-          <t>risc_haz_04</t>
+          <t>risc_rst_01</t>
         </is>
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>Control-flush cleanliness: instructions younger than a taken branch / jump / trap never produce architectural side effects (no register write, no memory request).</t>
+          <t>Reset re-assertion during outstanding data transactions (load/store granted but rvalid pending, incl. mid misaligned pair).</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr"/>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>sb, lsu_pas_mon</t>
+          <t>sys_ctrl_agent, lsu_agent, uvm_scoreboard</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="5" t="inlineStr">
         <is>
-          <t>risc_rf_00</t>
+          <t>risc_rst_02</t>
         </is>
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>x0 is hardwired to zero: reads always return 0 and writes to x0 are ignored (x0 has no flip-flops), even when a load targets x0.</t>
+          <t>Reset re-assertion during a multicycle DIV/REM or MULH execution, and during a branch-flush window.</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr"/>
       <c r="D53" s="5" t="inlineStr">
         <is>
-          <t>sb, rvfi_pas_mon</t>
+          <t>sys_ctrl_agent, uvm_scoreboard</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="5" t="inlineStr">
         <is>
-          <t>risc_rf_01</t>
+          <t>risc_env_00</t>
         </is>
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>All 31 general-purpose registers x1..x31 are implemented (FF register file resets to 0 at rst_ni==0) with 3 read ports and 2 write ports; reads happen in ID, writes from EX and WB.</t>
-        </is>
-      </c>
-      <c r="C54" s="5" t="inlineStr">
-        <is>
-          <t>Reset-zero is an implementation property of the FF-based RF in this repo - checked once at test start, not mandated by the ISA.</t>
-        </is>
-      </c>
+          <t>The TB includes its own instruction memory and data memory models working as OBI slaves. The instruction memory is pre-loaded with a generated or directed program before the core is enabled; the data memory is pre-loaded with a data pool. All memory words are deterministically initialized, so loads of unwritten locations are reproducible and match the golden model.</t>
+        </is>
+      </c>
+      <c r="C54" s="5" t="inlineStr"/>
       <c r="D54" s="5" t="inlineStr">
         <is>
-          <t>sb</t>
+          <t>if_agent (instr_mem_model), lsu_agent (data_mem_model), riscv_program</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="5" t="inlineStr">
         <is>
-          <t>risc_rst_00</t>
+          <t>risc_env_01</t>
         </is>
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>Reset re-assertion during an outstanding instruction-fetch transaction: core and TB slave both drop the transaction; after re-enabling, the core re-boots from boot_addr_i with a clean pipeline; no stale rvalid may be consumed after reset.</t>
-        </is>
-      </c>
-      <c r="C55" s="5" t="inlineStr">
-        <is>
-          <t>TB OBI slaves implement a reset that clears their outstanding queues.</t>
-        </is>
-      </c>
+          <t>OBI slave response features: per-transaction gnt delay (0..K), rvalid delay (1..L); operating modes: zero-wait, random, long-stall bursts, gnt-always-high; both buses configurable independently.</t>
+        </is>
+      </c>
+      <c r="C55" s="5" t="inlineStr"/>
       <c r="D55" s="5" t="inlineStr">
         <is>
-          <t>sys_ctrl_agent, if_agt, sb</t>
+          <t>if_agent, lsu_agent</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="5" t="inlineStr">
         <is>
-          <t>risc_rst_01</t>
+          <t>risc_env_02</t>
         </is>
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>Reset re-assertion during outstanding data transactions (load/store granted but rvalid pending, incl. mid misaligned pair).</t>
+          <t>Test teardown: at end of test all outstanding responses are delivered (memory drains), the retire stream is checked complete against expectations, and the final GPR + memory state is compared; a global watchdog timeout catches any hung core.</t>
         </is>
       </c>
       <c r="C56" s="5" t="inlineStr"/>
       <c r="D56" s="5" t="inlineStr">
         <is>
-          <t>sys_ctrl_agent, lsu_agt, sb</t>
+          <t>uvm_scoreboard, top_tb</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="5" t="inlineStr">
         <is>
-          <t>risc_rst_02</t>
+          <t>risc_scope_00</t>
         </is>
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>Reset re-assertion during a multicycle DIV/REM or MULH execution, and during a branch-flush window.</t>
-        </is>
-      </c>
-      <c r="C57" s="5" t="inlineStr"/>
+          <t>Features outside the verification goal - kept inactive (static tie-offs) or never generated, listed here only as constraints: C-extension internals (aligner/compressed decoder), CSR instructions and CSR state, interrupts, debug, sleep unit / wfi / elw, FPU and FP CSRs, CORE-V custom (PULP/CLUSTER) instructions and CSRs, atomics / PMP / user mode, performance counters, FENCE / ECALL / EBREAK / MRET.</t>
+        </is>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>No checkers or coverage are built for these.</t>
+        </is>
+      </c>
       <c r="D57" s="5" t="inlineStr">
-        <is>
-          <t>sys_ctrl_agent, sb</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="5" t="inlineStr">
-        <is>
-          <t>risc_env_00</t>
-        </is>
-      </c>
-      <c r="B58" s="5" t="inlineStr">
-        <is>
-          <t>The TB implements instruction memory and data memory models as OBI slaves (guideline Team1 Q5: the whole TB incl. memory is ours). The instruction memory is pre-loaded with a generated or directed program before enabling the core (compliant option (b) of Team4 Q5); the data memory is pre-loaded with a data pool. All memory words are deterministically initialized (loads of unwritten locations are reproducible and covered by the golden model).</t>
-        </is>
-      </c>
-      <c r="C58" s="5" t="inlineStr"/>
-      <c r="D58" s="5" t="inlineStr">
-        <is>
-          <t>if_agt (instr_mem_model), lsu_agt (data_mem_model), riscv_program</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="5" t="inlineStr">
-        <is>
-          <t>risc_env_01</t>
-        </is>
-      </c>
-      <c r="B59" s="5" t="inlineStr">
-        <is>
-          <t>OBI slave response generation features: per-transaction gnt delay (0..K), rvalid delay (1..L), operating modes: zero-wait, random, long-stall bursts, gnt-always-high; both buses independently configurable.</t>
-        </is>
-      </c>
-      <c r="C59" s="5" t="inlineStr"/>
-      <c r="D59" s="5" t="inlineStr">
-        <is>
-          <t>if_agt, lsu_agt</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="5" t="inlineStr">
-        <is>
-          <t>risc_env_02</t>
-        </is>
-      </c>
-      <c r="B60" s="5" t="inlineStr">
-        <is>
-          <t>Test teardown: at end of test all outstanding responses are delivered (memory drains), the retire stream is empty-checked against expectations, and the final GPR + memory state is compared; a global watchdog timeout catches any hung core.</t>
-        </is>
-      </c>
-      <c r="C60" s="5" t="inlineStr"/>
-      <c r="D60" s="5" t="inlineStr">
-        <is>
-          <t>sb, top_tb</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="5" t="inlineStr">
-        <is>
-          <t>risc_scope_00</t>
-        </is>
-      </c>
-      <c r="B61" s="5" t="inlineStr">
-        <is>
-          <t>Out of verification scope (guidelines): C-extension internals (aligner/compressed decoder), CSR instruction/state verification, interrupts, debug, sleep unit/wfi/elw, FPU and FP CSRs, COREV_PULP/COREV_CLUSTER custom instructions and CSRs, atomics/PMP/User-mode, performance counters, FENCE/ECALL/EBREAK/MRET. These appear in the plan ONLY as tie-offs, anti-checks, or illegal encodings - never as functional goals.</t>
-        </is>
-      </c>
-      <c r="C61" s="5" t="inlineStr">
-        <is>
-          <t>Mirrors template 'Features Not Supported' row.</t>
-        </is>
-      </c>
-      <c r="D61" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1745,7 +1672,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>Generate reset with random hold time and random de-assert phase relative to clk_i; apply single reset at test start and (in dedicated tests) re-assert mid-operation</t>
+          <t>Generate reset with random hold time and random de-assert phase relative to clk_i; apply a single reset at test start and (in dedicated tests) re-assert mid-operation</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
@@ -1767,7 +1694,7 @@
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>Randomize boot_addr_i across legal word-aligned memory window (low / middle / high addresses, incl. address-bit corner values)</t>
+          <t>Randomize boot_addr_i across the legal word-aligned memory window (low / middle / high addresses, incl. address-bit corner values)</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
@@ -1789,7 +1716,7 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Randomize mtvec_addr_i per test over 256B-aligned window (several distinct bases incl. different upper-byte values to catch base-bit bugs)</t>
+          <t>Randomize mtvec_addr_i per test over a 256B-aligned window (several distinct bases incl. different upper-byte values to catch base-bit bugs)</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
@@ -1806,12 +1733,12 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>fetch_enable_i: the first instruction fetch after reset de-assertion must not happen while fetch_enable_i==0; after fetch_enable_i has been 1 for at least one cycle (out of reset) fetching starts permanently, and the value of fetch_enable_i is ignored until the next reset. boot_addr_i/mtvec_addr_i/dm_*_addr_i/hart_id_i must stay stable once enabled.</t>
+          <t>fetch_enable_i: the first instruction fetch after reset de-assertion must not happen while fetch_enable_i==0; after fetch_enable_i has been 1 for at least one cycle (out of reset) fetching starts permanently, and the value of fetch_enable_i is ignored until the next reset. boot_addr_i / mtvec_addr_i / dm_*_addr_i / hart_id_i must stay stable once the core is enabled.</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Randomize the delay between reset de-assertion and fetch_enable_i rising (0,1,...,N cycles, N up toStress); keep fetch_enable_i high afterwards</t>
+          <t>Randomize the delay between reset de-assertion and fetch_enable_i rising (0,1,...,N cycles); keep fetch_enable_i high afterwards</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
@@ -1877,7 +1804,7 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Randomize rvalid latency 1..L cycles per transaction (L up toStress), incl. separating responses of two outstanding requests</t>
+          <t>Randomize rvalid latency 1..L cycles per transaction (L up to stress), incl. separating responses of two outstanding requests</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
@@ -1916,12 +1843,12 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Flush on taken jump (JAL/JALR are resolved in ID stage): the prefetch buffer and IF stage are flushed; the new PC request appears on the instruction-side memory interface in the same cycle the jump is in ID; with zero wait states the jump costs 2 cycles.</t>
+          <t>Flush on taken jump (JAL/JALR are resolved in the ID stage): the prefetch buffer and IF stage are flushed; the new PC request appears on the instruction-side memory interface in the same cycle the jump is in ID; with zero wait states the jump costs 2 cycles.</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Generate jumps forward/backward incl. small (+/- few words) and large offsets, link regs x0/x1/x5; JALR with odd immediate so target uses the &amp;~1 rule on a word-aligned address</t>
+          <t>Generate jumps forward/backward incl. small (+/- few words) and large offsets, link regs x0/x1/x5; JALR with odd immediate so the target uses the &amp;~1 rule on a word-aligned address</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
@@ -1938,7 +1865,7 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Flush on taken branch (resolved in EX stage): IF stage and ID stage are flushed; fetch restarts at the branch target; with zero wait states a taken branch costs 3 cycles; a not-taken branch costs 1 cycle (no stall).</t>
+          <t>Flush on taken branch (resolved in the EX stage): the IF stage and ID stage are flushed; fetch restarts at the branch target; with zero wait states a taken branch costs 3 cycles; a not-taken branch costs 1 cycle (no stall).</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
@@ -1982,7 +1909,7 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Stimulus constraint: all generated programs consist of 32-bit instructions only, word-aligned (no RVC encodings), with word-aligned branch/jump targets; programs are bounded and terminate at a defined end-of-program sentinel address recognized by the teardown. The aligner and compressed decoder are part of the never-tested C extension per guideline Team2 Q1 and are exercised only as pass-through hardware.</t>
+          <t>Stimulus constraint: all generated programs consist of 32-bit instructions only, word-aligned (no RVC encodings), with word-aligned branch/jump targets; programs are bounded and terminate at a defined end-of-program sentinel address recognized by the teardown. The aligner and compressed decoder belong to the never-tested C extension and are exercised only as pass-through hardware.</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
@@ -2004,7 +1931,7 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Data OBI handshake: data_req_o is raised for load/store and must stay high until data_gnt_i is sampled high; data_addr_o, data_we_o, data_be_o, data_wdata_o are send together with the request and must stay stable while req==1 &amp;&amp; gnt==0.</t>
+          <t>Data OBI handshake: data_req_o is raised for load/store and must stay high until data_gnt_i is sampled high; data_addr_o, data_we_o, data_be_o, data_wdata_o are sent together with the request and must stay stable while req==1 &amp;&amp; gnt==0.</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
@@ -2057,7 +1984,7 @@
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>Generate lw/sw at all 4 offsets, lh/sh at all 4 offsets, lb/lbu/lh/lhu/sb at all 4 offsets</t>
+          <t>Generate lw/sw at all 4 offsets, lh/sh at all 4 offsets, lb/lbu/sb at all 4 offsets</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
@@ -2074,12 +2001,12 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Misaligned handling: the LSU never raises address-misaligned exceptions. A word load/store at addr[1:0]!=00, or a halfword at addr[1:0]==11, is performed as TWO bus transactions; the transfer for the lowest address is issued first, followed by (aligned base+4) with the complementary byte-enables; the core spends 2 cycles each in EX and WB per part and merges the response data. All other offsets need a single transaction.</t>
+          <t>Misaligned handling: the LSU never raises address-misaligned exceptions. A word load/store at addr[1:0]!=00, or a halfword at addr[1:0]==11, is performed as TWO bus transactions; the transfer for the lowest address is issued first, followed by (aligned base+4) with the complementary byte-enables; the memory transfers for the two parts are merged by the core into one load/store view. All other offsets need a single transaction.</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>Generate misaligned lw/sw at offsets 1,2,3 and lh/sh at offset 3 (crossing) and offset 1,2 (non-crossing), incl. back-to-back misaligned pairs</t>
+          <t>Generate misaligned lw/sw at offsets 1,2,3 and lh/sh at offset 3 (crossing) and offsets 1,2 (non-crossing), incl. back-to-back misaligned pairs</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
@@ -2118,7 +2045,7 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>Load data alignment and extension: LB/LH sign-extend the addressed byte/halfword; LBU/LHU zero-extend; LW returns the full word; for misaligned accesses the two response words are assembled (first-response low bytes kept in rdata_q, combined with second response) according to the address offset.</t>
+          <t>Load data alignment and extension: LB/LH sign-extend the addressed byte/halfword; LBU/LHU zero-extend; LW returns the full word; for misaligned accesses the two response words are assembled (first-response low bytes kept in rdata_q, combined with the second response) according to the address offset.</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
@@ -2140,7 +2067,7 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>Memory consistency: in-order data responses + single hart imply a load must observe the value of the most recent previously-issued store to the same byte address; the TB memory model commits a store at its rvalid and never reorders.</t>
+          <t>Memory consistency: in-order data responses and a single hart imply a load must observe the value of the most recent previously-issued store to the same byte address; the TB memory model commits a store at its rvalid and never reorders.</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
@@ -2184,7 +2111,7 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>All RV32I base instructions are legal and must execute correctly: LUI, AUIPC, JAL, JALR, BEQ, BNE, BLT, BGE, BLTU, BGEU, LB, LH, LW, LBU, LHU, SB, SH, SW, ADDI, SLTI, SLTIU, XORI, ORI, ANDI, SLLI, SRLI, SRAI, ADD, SUB, SLL, SLT, SLTU, XOR, SRL, SRA, OR, AND. (FENCE/FENCE.I/ECALL/EBREAK are part of the base but are excluded from stimulus per guideline Team4 Q2.)</t>
+          <t>All RV32I base instructions are legal and must execute correctly: LUI, AUIPC, JAL, JALR, BEQ, BNE, BLT, BGE, BLTU, BGEU, LB, LH, LW, LBU, LHU, SB, SH, SW, ADDI, SLTI, SLTIU, XORI, ORI, ANDI, SLLI, SRLI, SRAI, ADD, SUB, SLL, SLT, SLTU, XOR, SRL, SRA, OR, AND. (FENCE / FENCE.I / ECALL / EBREAK are part of the base ISA but are omitted from the generated stimulus.)</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
@@ -2228,16 +2155,15 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>Illegal instruction detection (verified against cv32e40p_decoder.sv illegal_insn conditions): any encoding undefined for the configured parameter set raises an illegal instruction exception, including:
+          <t>Illegal instruction detection within the RV32I/M opcode space (verified against cv32e40p_decoder.sv illegal_insn conditions): any undefined encoding raises an illegal instruction exception, including:
 (a) undefined major opcodes;
-(b) legal major opcode with undefined funct3/funct7 combination;
-(c) reserved shift encodings: OP-IMM/OP with funct3=001/101 and imm[11:5] (funct7) other than 0000000 or 0100000;
-(d) F / D / A major opcodes (FPU=0, atomics removed); (e) SYSTEM/CSR instructions accessing unimplemented CSR addresses; (f) CORE-V custom opcode spaces (incl. 0x0B, 0x2B, 0x5B, 0x7B) while COREV_PULP=0 / COREV_CLUSTER=0.</t>
+(b) a legal major opcode with an undefined funct3/funct7 combination;
+(c) reserved shift encodings: OP-IMM/OP with funct3=001/101 and imm[11:5] (funct7) other than 0000000 or 0100000.</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>Generate items from each illegal category (a)-(f) with randomized filler bits; inject at random stream positions</t>
+          <t>Generate items from each illegal category (a)-(c) with randomized filler bits; inject at random stream positions</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
@@ -2249,7 +2175,7 @@
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>risc_dec_04</t>
+          <t>risc_dec_03</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
@@ -2271,17 +2197,17 @@
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>risc_dec_05</t>
+          <t>risc_dec_04</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>Excluded from stimulus per guidelines (Team2 Q5, Team3, Team4 Q2/Q3, Team5 Q3): FENCE, FENCE.I, ECALL, EBREAK, WFI, MRET and all CSR instructions; interrupt and debug traffic; compressed instructions; all FPU/PULP/atomic instructions (they only appear as illegal-encoding injections, never as legal flow).</t>
+          <t>Omitted from stimulus (generation constraint): FENCE, FENCE.I, ECALL, EBREAK, WFI, MRET and all CSR instructions; interrupt and debug traffic; compressed instructions; all FPU / CORE-V custom / atomic instructions (including their opcodes as partial encodings).</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>not generated (except as illegal-category injections for risc_dec_02)</t>
+          <t>not generated</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
@@ -2298,7 +2224,7 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>Integer computational instructions (ADD/SUB/AND/OR/XOR/SLL/SRL/SRA/SLT/SLTU + I-forms, LUI, AUIPC) produce their result in 1 cycle; the EX-&gt;ID forwarding path provides a 0-cycle penalty for a back-to-back dependent ALU instruction; SLT/SLTU distinguish signed vs unsigned compare and SLTIU compares rs1 unsigned against the sign-extended immediate (per RISC-V spec).</t>
+          <t>Integer computational instructions (ADD/SUB/AND/OR/XOR/SLL/SRL/SRA/SLT/SLTU + I-forms, LUI, AUIPC) produce their result in 1 cycle; the EX-&gt;ID forwarding path gives a 0-cycle penalty for a back-to-back dependent ALU instruction; SLT/SLTU distinguish signed vs unsigned compare and SLTIU compares rs1 unsigned against the sign-extended immediate (per the RISC-V spec).</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
@@ -2320,7 +2246,7 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>Shifts use a single-cycle barrel shifter; shift amount shamt is operand_b[4:0] (reg form) or imm[4:0]; SRA/SRAI replicate the sign bit; SLL/SRL shift in zeros. shamt=0 leaves the operand unchanged.</t>
+          <t>Shifts use a single-cycle barrel shifter; the shift amount shamt is operand_b[4:0] (register form) or imm[4:0]; SRA/SRAI replicate the sign bit; SLL/SRL shift in zeros. shamt=0 leaves the operand unchanged.</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
@@ -2342,7 +2268,7 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>LUI writes imm[31:12]&lt;&lt;12; AUIPC writes PC + (imm&lt;&lt;12) - the value depends on the current PC (position-dependent behavior).</t>
+          <t>LUI writes imm[31:12]&lt;&lt;12; AUIPC writes PC + (imm&lt;&lt;12) - the result depends on the current PC (position-dependent behavior).</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
@@ -2369,7 +2295,7 @@
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>Generate MUL with corner operands (0, 1, -1, INT_MIN, INT_MAX, random 16x16 bit patterns that stress partial products)</t>
+          <t>Generate MUL with corner operands (0, 1, -1, INT_MIN, INT_MAX, random 16x16-bit patterns that stress partial products)</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
@@ -2408,7 +2334,7 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>DIV/DIVU/REM/REMU are iterative with early termination: latency is 3..35 cycles depending on the number of leading zeros of operand b (divisor); minimum 3 cycles when the divisor has no leading zeros (e.g. 0x80000000), maximum 35 when the divisor is 0; EX stalls meanwhile.</t>
+          <t>DIV/DIVU/REM/REMU are iterative with early termination: latency is 3..35 cycles depending on the number of leading zeros of operand b (the divisor); minimum 3 cycles when the divisor has no leading zeros (e.g. 0x80000000), maximum 35 when the divisor is 0; EX stalls meanwhile.</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
@@ -2430,7 +2356,7 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>Special division results per RISC-V spec: Divide-by-zero -&gt; quotient = -1 (all ones) for DIV/DIVU; remainder = dividend for REM/REMU. Signed overflow (DIV -2^31 / -1) -&gt; quotient = -2^31, REM -2^31 / -1 -&gt; 0. REM sign follows the dividend; REMU is unsigned.</t>
+          <t>Special division results per the RISC-V spec: divide-by-zero -&gt; quotient = -1 (all ones) for DIV/DIVU; remainder = dividend for REM/REMU. Signed overflow (DIV -2^31 / -1) -&gt; quotient = -2^31, REM -2^31 / -1 -&gt; 0. The REM sign follows the dividend; REMU is unsigned.</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
@@ -2452,7 +2378,7 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>A multicycle instruction (MULH/DIV/REM) that is older than a taken branch always completes and writes back normally even if the flush of younger instructions happens in the same window (answer to open guideline question Team4 Q4, resolved from databook pipeline chapter and rtl: only IF/ID - i.e. younger instructions - are flushed).</t>
+          <t>A multicycle instruction (MULH/DIV/REM) that is older than a taken branch always completes and writes back normally, even when the flush of the younger path lands in the same window - only IF/ID (the younger stages) are flushed.</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
@@ -2474,7 +2400,7 @@
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>RAW forwarding: ALU/MUL/DIV results in EX are forwarded to ID-stage operands (ports a and b), giving 0-cycle penalty for back-to-back dependent instructions; the consumer reads correct producer values at distance 1, 2, 3.</t>
+          <t>RAW forwarding: ALU/MUL/DIV results in EX are forwarded to ID-stage operands (ports a and b), giving a 0-cycle penalty for back-to-back dependent instructions; the consumer reads correct producer values at distance 1, 2, 3.</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
@@ -2540,12 +2466,12 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>WAW write-port arbitration: a load in WB and a younger ALU/MUL/DIV instruction in EX may write the same rd in the same cycle; the register file resolves it with port-b (EX) priority, i.e. the architecturally younger instruction wins (open guideline question Team4 Q6, answered directly from rtl cv32e40p_register_file_ff.sv: we_b checked before we_a).</t>
+          <t>WAW write-port arbitration: a load in WB and a younger ALU/MUL/DIV instruction in EX may write the same rd in the same cycle; the register file resolves it with port-b (EX) priority, i.e. the architecturally younger instruction wins (verified in rtl cv32e40p_register_file_ff.sv: the we_b write is checked before we_a).</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>Generate lw rd,&lt;-mem followed at distance 1..3 by an ALU/MUL/DIV op writing the same rd (and the reverse order is impossible); sweep rd incl. x0 exclusion semantics; include a misaligned-load producer variant (pair completes in WB while younger EX write lands)</t>
+          <t>Generate lw rd,&lt;-mem followed at distance 1..3 by an ALU/MUL/DIV op writing the same rd; sweep rd incl. x0 exclusion semantics; include a misaligned-load producer variant (pair completes in WB while the younger EX write lands)</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
@@ -2562,7 +2488,7 @@
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>All 31 general-purpose registers x1..x31 are implemented (FF register file resets to 0 at rst_ni==0) with 3 read ports and 2 write ports; reads happen in ID, writes from EX and WB.</t>
+          <t>All 31 general-purpose registers x1..x31 are implemented (the FF register file resets to 0 at rst_ni==0) with 3 read ports and 2 write ports; reads happen in ID, writes from EX and WB.</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
@@ -2650,12 +2576,12 @@
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>OBI slave response generation features: per-transaction gnt delay (0..K), rvalid delay (1..L), operating modes: zero-wait, random, long-stall bursts, gnt-always-high; both buses independently configurable.</t>
+          <t>OBI slave response features: per-transaction gnt delay (0..K), rvalid delay (1..L); operating modes: zero-wait, random, long-stall bursts, gnt-always-high; both buses configurable independently.</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>Seeds sweeping: short/medium/long delay distributions, alternating fast/slow window lengths, simultaneous stalls on both buses</t>
+          <t>Seed sweeping: short/medium/long delay distributions, alternating fast/slow window lengths, simultaneous stalls on both buses</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
@@ -2678,7 +2604,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E51"/>
+  <dimension ref="A1:E47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20.7" customWidth="1" min="1" max="1"/>
@@ -2747,7 +2673,7 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>SVA inside if_pas / lsu_pas</t>
+          <t>SVA inside if_passive_agent.output_monitor / lsu_passive_agent.output_monitor</t>
         </is>
       </c>
     </row>
@@ -2774,7 +2700,7 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>SVA via if_pas_mon sampling instr_addr_o of 1st granted request after fetch_enable</t>
+          <t>SVA inside if_passive_agent.output_monitor, sampling instr_addr_o of the 1st granted request after fetch_enable</t>
         </is>
       </c>
     </row>
@@ -2801,7 +2727,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>sb / if_pas_mon observing fetch redirect</t>
+          <t>uvm_scoreboard / if_passive_agent observing the fetch redirect</t>
         </is>
       </c>
     </row>
@@ -2813,7 +2739,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>fetch_enable_i: the first instruction fetch after reset de-assertion must not happen while fetch_enable_i==0; after fetch_enable_i has been 1 for at least one cycle (out of reset) fetching starts permanently, and the value of fetch_enable_i is ignored until the next reset. boot_addr_i/mtvec_addr_i/dm_*_addr_i/hart_id_i must stay stable once enabled.</t>
+          <t>fetch_enable_i: the first instruction fetch after reset de-assertion must not happen while fetch_enable_i==0; after fetch_enable_i has been 1 for at least one cycle (out of reset) fetching starts permanently, and the value of fetch_enable_i is ignored until the next reset. boot_addr_i / mtvec_addr_i / dm_*_addr_i / hart_id_i must stay stable once the core is enabled.</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
@@ -2828,7 +2754,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>SVA via sys_ctrl_agent / if_pas_mon</t>
+          <t>SVA inside if_passive_agent.output_monitor</t>
         </is>
       </c>
     </row>
@@ -2840,383 +2766,302 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>With irq_i tied to 0, no interrupt may ever be taken: irq_ack_o must stay 0 for the whole simulation.</t>
+          <t>Primary outputs of cv32e40p_top must never be X/Z after reset de-assertion while the core is clocked: instr_req_o, instr_addr_o, data_req_o, data_we_o, data_be_o, data_addr_o, data_wdata_o (when driven).</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>check that irq_ack_o is constantly 0 (and irq_id_o stable) during the entire simulation</t>
+          <t>check no X on primary outputs at every clk_i edge when rst_ni==1</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>sys_no_irq_prop</t>
+          <t>outputs_no_x_prop</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>SVA</t>
+          <t>SVA ($isunknown) inside both passive output monitors</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>risc_sys_08</t>
+          <t>risc_if_00</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>With debug_req_i tied to 0 and no ebreak stimulus, the core must never enter Debug Mode: debug_halted_o must stay 0 after startup. debug_havereset_o / debug_running_o / debug_halted_o are mutually exclusive (exactly one asserted at any time); debug_havereset_o is set during reset and clears a few cycles after reset de-assert with fetch_enable_i high.</t>
+          <t>Instruction fetch OBI handshake: instr_req_o is raised for a fetch and must stay high until instr_gnt_i is sampled high for one cycle (request persistence - a request must never be retracted or its address changed once issued).</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>check mutual exclusivity of debug_havereset_o / debug_running_o / debug_halted_o and that debug_halted_o==0 constantly</t>
+          <t>check that instr_req_o stays asserted and instr_addr_o stays stable in every cycle with req==1 &amp;&amp; gnt==0</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>debug_status_excl_prop</t>
+          <t>if_obi_req_persistence_prop, if_obi_addr_stable_prop</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>SVA</t>
+          <t>SVA inside if_passive_agent.output_monitor</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>risc_sys_09</t>
+          <t>risc_if_01</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>core_sleep_o must stay 0 for the whole simulation: no wfi and no cv.elw are ever generated (out of scope), so the internal clock is never gated after fetch_enable_i.</t>
+          <t>instr_req_o must not combinationally depend on instr_rvalid_i (OBI: no rvalid-&gt;req dependency); instr_gnt_i may be high even when there is no request, which must not cause any spurious side effect.</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>check that core_sleep_o is constantly 0</t>
+          <t>check that granted-count and valid-count match over the whole test: #(req&amp;&amp;gnt) == #(rvalid) by end of test (no request swallowed, no phantom response accepted)</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>sys_no_sleep_prop</t>
+          <t>if_obi_trans_match_prop</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>SVA</t>
+          <t>if_passive_agent transaction counters, compared at end of test</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>risc_sys_10</t>
+          <t>risc_if_02</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Primary outputs of cv32e40p_top must never be X/Z after reset de-assertion while the core is clocked: instr_req_o, instr_addr_o, data_req_o, data_we_o, data_be_o, data_addr_o, data_wdata_o (when driven).</t>
+          <t>Response phase: instr_rvalid_i is high for exactly one cycle per granted request; instr_rdata_i is sampled in that cycle. Responses must arrive in issue order (master point of view), possibly one or more cycles after grant; the IF interface can have up to DEPTH=2 outstanding requests.</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>check no X on primary outputs at every clk_i edge when rst_ni==1</t>
+          <t>check environment guarantee assertions: rvalid only when a granted outstanding request exists; exactly one rvalid pulse per granted request; rdata stable during its rvalid cycle; responses in issue order</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>outputs_no_x_prop</t>
+          <t>if_obi_slave_protocol_prop</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>SVA $isunknown in if_pas / lsu_pas</t>
+          <t>Assertions inside if_agent (instr_mem_model) as an environment self-check</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>risc_if_00</t>
+          <t>risc_if_03</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Instruction fetch OBI handshake: instr_req_o is raised for a fetch and must stay high until instr_gnt_i is sampled high for one cycle (request persistence - a request must never be retracted or its address changed once issued).</t>
+          <t>Back-to-back fetches: while the prefetch FIFO drains, a new instr_req_o may be issued in the cycle immediately following a gnt; a continuous request stream must be sustained.</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>check that instr_req_o stays asserted and instr_addr_o stays stable in every cycle with req==1 &amp;&amp; gnt==0</t>
+          <t>check functional continuity of the fetch stream into the scoreboard instruction queue (no duplicated / lost fetch word observed at retire time)</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>if_obi_req_persistence_prop, if_obi_addr_stable_prop</t>
+          <t>sb_fetch_stream_consistent</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>SVA inside if_pas_mon</t>
+          <t>uvm_scoreboard (if_passive_agent transaction log vs rvfi_monitor PCs)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>risc_if_01</t>
+          <t>risc_if_05</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>instr_req_o must not combinationally depend on instr_rvalid_i (OBI: no rvalid-&gt;req dependency); instr_gnt_i may be high even when there is no request, which must not cause any spurious side effect.</t>
+          <t>Flush on taken jump (JAL/JALR are resolved in the ID stage): the prefetch buffer and IF stage are flushed; the new PC request appears on the instruction-side memory interface in the same cycle the jump is in ID; with zero wait states the jump costs 2 cycles.</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>check that granted-count and valid-count match over the whole test: #(req&amp;&amp;gnt) == #(rvalid) by end of test (no request swallowed, no phantom response accepted)</t>
+          <t>check via the scoreboard that the retired-PC stream follows exactly: fall-through PCs never retire after a jump; the target PC retires as the jump successor (JAL: PC+imm; JALR: (rs1+imm) &amp; ~1); the link register rd == PC+4</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>if_obi_trans_match_prop</t>
+          <t>sb_pc_flow_match, sb_jump_link_match</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>if_pas_mon counters + end-of-test compare</t>
+          <t>uvm_scoreboard (rvfi_monitor + ref_model)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>risc_if_02</t>
+          <t>risc_if_06</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Response phase: instr_rvalid_i is high for exactly one cycle per granted request; instr_rdata_i is sampled in that cycle. Responses must arrive in issue order (master point of view), possibly one or more cycles after grant; the IF interface can have up to DEPTH=2 outstanding requests.</t>
+          <t>Flush on taken branch (resolved in the EX stage): the IF stage and ID stage are flushed; fetch restarts at the branch target; with zero wait states a taken branch costs 3 cycles; a not-taken branch costs 1 cycle (no stall).</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>check environment guarantee assertions: rvalid only when a granted outstanding request exists; exactly one rvalid pulse per granted request; rdata stable during its rvalid cycle; responses in issue order</t>
+          <t>check via the scoreboard that instructions fetched after a taken branch on the fall-through path retire no architectural effect, and the retired-PC stream continues at the branch target (PC+imm)</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>if_obi_slave_protocol_prop</t>
+          <t>sb_pc_flow_match, sb_flush_clean</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>Assertions inside the OBI slave (environment self-check)</t>
+          <t>uvm_scoreboard</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>risc_if_03</t>
+          <t>risc_if_07</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Back-to-back fetches: while the prefetch FIFO drains, a new instr_req_o may be issued in the cycle immediately following a gnt; a continuous request stream must be sustained.</t>
+          <t>Flush on trap (illegal instruction): the pipeline is flushed and fetch restarts at the mtvec base address; handler code at the base continues normally afterwards.</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>check functional continuity of the fetch stream into the scoreboard instruction queue (no duplicated / lost fetch word observed at retire time)</t>
+          <t>check that after the trapped instruction, the next retired PC equals the mtvec base and subsequent retired PCs follow the handler program</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>sb_fetch_stream_consistent</t>
+          <t>sb_trap_redirect</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>sb (via if_pas_mon transaction log vs rvfi PCs)</t>
+          <t>uvm_scoreboard (via rvfi_monitor), cf. risc_sys_04 / risc_dec_02</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>risc_if_05</t>
+          <t>risc_if_09</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Flush on taken jump (JAL/JALR are resolved in ID stage): the prefetch buffer and IF stage are flushed; the new PC request appears on the instruction-side memory interface in the same cycle the jump is in ID; with zero wait states the jump costs 2 cycles.</t>
+          <t>No instruction-address-misaligned exception exists in this core (the C extension is always enabled), so instruction fetch must never cause a trap; any trap observed on a legal stream is a bug.</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>check via scoreboard that the retired-PC stream follows exactly: fall-through PCs never retire after a jump; target PC retires as the jump successor (JAL: PC+imm; JALR: (rs1+imm) &amp; ~1); link register rd == PC+4</t>
+          <t>check that no trap redirect occurs on streams containing only legal instructions</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>sb_pc_flow_match, sb_jump_link_match</t>
+          <t>sb_no_unexpected_trap</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>sb (rvfi_pas_mon + reference model)</t>
+          <t>uvm_scoreboard</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>risc_if_06</t>
+          <t>risc_lsu_00</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Flush on taken branch (resolved in EX stage): IF stage and ID stage are flushed; fetch restarts at the branch target; with zero wait states a taken branch costs 3 cycles; a not-taken branch costs 1 cycle (no stall).</t>
+          <t>Data OBI handshake: data_req_o is raised for load/store and must stay high until data_gnt_i is sampled high; data_addr_o, data_we_o, data_be_o, data_wdata_o are sent together with the request and must stay stable while req==1 &amp;&amp; gnt==0.</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>check via scoreboard that instructions fetched after a taken branch on the fall-through path retire no architectural effect, and the retired-PC stream continues at the branch target (PC+imm)</t>
+          <t>check request persistence and address/control/write-data stability during non-granted cycles</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>sb_pc_flow_match, sb_flush_clean</t>
+          <t>lsu_obi_req_persistence_prop, lsu_obi_stable_prop</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>sb</t>
+          <t>SVA inside lsu_passive_agent.output_monitor</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>risc_if_07</t>
+          <t>risc_lsu_01</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>Flush on trap (illegal instruction): the pipeline is flushed and fetch restarts at the mtvec base address; handler code at the base continues normally afterwards.</t>
+          <t>Response phase (data side): data_rvalid_i is high for exactly one cycle per granted request and terminates both read and write transactions (for stores data_rdata_i is meaningless). Responses are in issue order; the data interface supports up to 2 outstanding transactions; when responses lag, the core applies back-pressure (EX/WB stall) instead of issuing further requests.</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>check that after the trapped instruction, the next retired PC equals the mtvec base and subsequent retired PCs follow the handler program</t>
+          <t>check environment guarantees (one rvalid per grant, in-order, no rvalid without outstanding) and that effectively never more than 2 outstanding exist on the data bus</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>sb_trap_redirect</t>
+          <t>lsu_obi_slave_protocol_prop, lsu_max_outstanding_prop</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>sb (rvfi_pas_mon), cf. risc_sys_04 / risc_dec_03</t>
+          <t>env assertions inside lsu_agent + lsu_passive_agent counter</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>risc_if_09</t>
+          <t>risc_lsu_03</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
-        <is>
-          <t>No instruction-address-misaligned exception exists in this core (the C extension is always enabled), so instruction fetch must never cause a trap; any trap observed on a legal stream is a bug.</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
-          <t>check that no trap redirect occurs on streams containing only legal instructions</t>
-        </is>
-      </c>
-      <c r="D18" s="5" t="inlineStr">
-        <is>
-          <t>sb_no_unexpected_trap</t>
-        </is>
-      </c>
-      <c r="E18" s="5" t="inlineStr">
-        <is>
-          <t>sb</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="5" t="inlineStr">
-        <is>
-          <t>risc_lsu_00</t>
-        </is>
-      </c>
-      <c r="B19" s="5" t="inlineStr">
-        <is>
-          <t>Data OBI handshake: data_req_o is raised for load/store and must stay high until data_gnt_i is sampled high; data_addr_o, data_we_o, data_be_o, data_wdata_o are send together with the request and must stay stable while req==1 &amp;&amp; gnt==0.</t>
-        </is>
-      </c>
-      <c r="C19" s="5" t="inlineStr">
-        <is>
-          <t>check request persistence and address/control/write-data stability during non-granted cycles</t>
-        </is>
-      </c>
-      <c r="D19" s="5" t="inlineStr">
-        <is>
-          <t>lsu_obi_req_persistence_prop, lsu_obi_stable_prop</t>
-        </is>
-      </c>
-      <c r="E19" s="5" t="inlineStr">
-        <is>
-          <t>SVA inside lsu_pas_mon</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="5" t="inlineStr">
-        <is>
-          <t>risc_lsu_01</t>
-        </is>
-      </c>
-      <c r="B20" s="5" t="inlineStr">
-        <is>
-          <t>Response phase (data side): data_rvalid_i is high for exactly one cycle per granted request and terminates both read and write transactions (for stores data_rdata_i is meaningless). Responses are in issue order; the data interface supports up to 2 outstanding transactions; when responses lag, the core applies back-pressure (EX/WB stall) instead of issuing further requests.</t>
-        </is>
-      </c>
-      <c r="C20" s="5" t="inlineStr">
-        <is>
-          <t>check environment guarantees (one rvalid per grant, in-order, no rvalid without outstanding) and that effectively never more than 2 outstanding exist on the data bus</t>
-        </is>
-      </c>
-      <c r="D20" s="5" t="inlineStr">
-        <is>
-          <t>lsu_obi_slave_protocol_prop, lsu_max_outstanding_prop</t>
-        </is>
-      </c>
-      <c r="E20" s="5" t="inlineStr">
-        <is>
-          <t>env assertions + lsu_pas_mon counter</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="5" t="inlineStr">
-        <is>
-          <t>risc_lsu_03</t>
-        </is>
-      </c>
-      <c r="B21" s="5" t="inlineStr">
         <is>
           <t>Byte-enable generation per access type and address (from rtl cv32e40p_load_store_unit.sv):
 SW: addr[1:0]=00-&gt;4'b1111; misaligned first beat 01-&gt;1110, 10-&gt;1100, 11-&gt;1000; second beat 01-&gt;0001, 10-&gt;0011, 11-&gt;0111.
@@ -3225,833 +3070,805 @@
 Only these patterns may ever appear on data_be_o.</t>
         </is>
       </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>check data_be_o is one of the legal patterns for the current access-type/address/phase on every granted data transaction</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>lsu_be_legal_prop</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>SVA/LUT check in lsu_passive_agent.output_monitor (access context taken from the monitor)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>risc_lsu_04</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Misaligned handling: the LSU never raises address-misaligned exceptions. A word load/store at addr[1:0]!=00, or a halfword at addr[1:0]==11, is performed as TWO bus transactions; the transfer for the lowest address is issued first, followed by (aligned base+4) with the complementary byte-enables; the memory transfers for the two parts are merged by the core into one load/store view. All other offsets need a single transaction.</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>check that misaligned word/halfword accesses produce exactly two OBI transactions: first beat address == original aligned address with phase-1 be, second beat address == +4 with phase-2 be, and that NO trap redirect happens; check the final loaded value and stored bytes match the golden model</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>lsu_misaligned_order_prop, sb_load_result_match, sb_no_exc_on_misaligned</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>SVA ordering check in lsu_passive_agent + uvm_scoreboard value check</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>risc_lsu_05</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Store data alignment: data_wdata_o is rotated by wdata_offset = addr[1:0] - reg_offset[1:0] (rtl formula), i.e. 01-&gt;{wdata[23:0],wdata[31:24]}, 10-&gt;{wdata[15:0],wdata[31:16]}, 11-&gt;{wdata[7:0],wdata[31:8]}; the memory applies data_be_o lanes only.</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>check stored bytes in the memory model equal the register content placed at the correct lanes (end-of-test memory compare + store-&gt;load readback within the test)</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>sb_store_mem_match</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>uvm_scoreboard vs golden memory model</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>risc_lsu_06</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Load data alignment and extension: LB/LH sign-extend the addressed byte/halfword; LBU/LHU zero-extend; LW returns the full word; for misaligned accesses the two response words are assembled (first-response low bytes kept in rdata_q, combined with the second response) according to the address offset.</t>
+        </is>
+      </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>check data_be_o is one of the legal patterns for the current access-type/address/phase on every granted data transaction</t>
+          <t>check every retired load: rd == golden sign/zero-extended value computed from the memory image at the effective address (incl. misaligned reassembly)</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>lsu_be_legal_prop</t>
+          <t>sb_load_result_match</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>SVA/lut check in lsu_pas_mon (needs access context from monitor)</t>
+          <t>uvm_scoreboard (golden RV32IM model)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>risc_lsu_04</t>
+          <t>risc_lsu_07</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>Misaligned handling: the LSU never raises address-misaligned exceptions. A word load/store at addr[1:0]!=00, or a halfword at addr[1:0]==11, is performed as TWO bus transactions; the transfer for the lowest address is issued first, followed by (aligned base+4) with the complementary byte-enables; the core spends 2 cycles each in EX and WB per part and merges the response data. All other offsets need a single transaction.</t>
+          <t>Memory consistency: in-order data responses and a single hart imply a load must observe the value of the most recent previously-issued store to the same byte address; the TB memory model commits a store at its rvalid and never reorders.</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>check that misaligned word/halfword accesses produce exactly two OBI transactions: first beat address == original aligned address with phase-1 be, second beat address == +4 with phase-2 be, and that NO trap redirect happens; check final loaded value and stored bytes match the golden model</t>
+          <t>check store-&gt;load same-address readback throughout the test (shadow memory in the scoreboard)</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>lsu_misaligned_order_prop, sb_load_result_match, sb_no_exc_on_misaligned</t>
+          <t>sb_mem_consistency</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>SVA order check + scoreboard value check</t>
+          <t>uvm_scoreboard shadow memory</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>risc_lsu_05</t>
+          <t>risc_lsu_08</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>Store data alignment: data_wdata_o is rotated by wdata_offset = addr[1:0] - reg_offset[1:0] (rtl formula), i.e. 01-&gt;{wdata[23:0],wdata[31:24]}, 10-&gt;{wdata[15:0],wdata[31:16]}, 11-&gt;{wdata[7:0],wdata[31:8]}; the memory applies data_be_o lanes only.</t>
+          <t>Flushed instructions must not affect the data bus: loads/stores younger than a taken branch, jump, or trap (still in IF/ID) are killed before their request phase - no spurious data_req_o from flushed instructions may appear.</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>check stored bytes in the memory model equal the register content placed at the correct lanes (end-of-test memory compare + store-&gt;load readback within test)</t>
+          <t>check that the data-bus transaction stream matches exactly the loads/stores that retire per the reference model (no extra, no missing transactions)</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>sb_store_mem_match</t>
+          <t>sb_lsu_trans_stream_match</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>sb vs golden memory model</t>
+          <t>uvm_scoreboard (lsu_passive_agent log vs ref_model)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>risc_lsu_06</t>
+          <t>risc_dec_00</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>Load data alignment and extension: LB/LH sign-extend the addressed byte/halfword; LBU/LHU zero-extend; LW returns the full word; for misaligned accesses the two response words are assembled (first-response low bytes kept in rdata_q, combined with second response) according to the address offset.</t>
+          <t>All RV32I base instructions are legal and must execute correctly: LUI, AUIPC, JAL, JALR, BEQ, BNE, BLT, BGE, BLTU, BGEU, LB, LH, LW, LBU, LHU, SB, SH, SW, ADDI, SLTI, SLTIU, XORI, ORI, ANDI, SLLI, SRLI, SRAI, ADD, SUB, SLL, SLT, SLTU, XOR, SRL, SRA, OR, AND. (FENCE / FENCE.I / ECALL / EBREAK are part of the base ISA but are omitted from the generated stimulus.)</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>check every retired load: rd == golden sign/zero-extended value computed from memory image at the effective address (incl. misaligned reassembly)</t>
+          <t>check every retired RV32I instruction against the golden model: rd value, memory effects, and next-PC</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>sb_load_result_match</t>
+          <t>sb_rv32i_result_match</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>sb (golden RV32IM model)</t>
+          <t>uvm_scoreboard (rvfi_monitor vs ref_model)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>risc_lsu_07</t>
+          <t>risc_dec_01</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>Memory consistency: in-order data responses + single hart imply a load must observe the value of the most recent previously-issued store to the same byte address; the TB memory model commits a store at its rvalid and never reorders.</t>
+          <t>All 8 RV32M instructions are legal and must execute correctly: MUL, MULH, MULHSU, MULHU, DIV, DIVU, REM, REMU.</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>check store-&gt;load same-address readback throughout the test (shadow memory in scoreboard)</t>
+          <t>check every retired RV32M instruction against the golden model (rd value and timing class)</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>sb_mem_consistency</t>
+          <t>sb_rv32m_result_match</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>sb</t>
+          <t>uvm_scoreboard</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>risc_lsu_08</t>
+          <t>risc_dec_02</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>Flushed instructions must not affect the data bus: loads/stores younger than a taken branch, jump, or trap (still in IF/ID) are killed before their request phase - no spurious data_req_o from flushed instructions may appear.</t>
+          <t>Illegal instruction detection within the RV32I/M opcode space (verified against cv32e40p_decoder.sv illegal_insn conditions): any undefined encoding raises an illegal instruction exception, including:
+(a) undefined major opcodes;
+(b) a legal major opcode with an undefined funct3/funct7 combination;
+(c) reserved shift encodings: OP-IMM/OP with funct3=001/101 and imm[11:5] (funct7) other than 0000000 or 0100000.</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>check that the data-bus transaction stream matches exactly the loads/stores that retire per the reference model (no extra, no missing transactions)</t>
+          <t>check that each injected illegal encoding is detected: the instruction retires to trap (no rd write, no memory request produced by it) and fetch redirects to mtvec base</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>sb_lsu_trans_stream_match</t>
+          <t>sb_illegal_trap, exc_trap_base_prop</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>sb (lsu_pas_mon log vs ref model)</t>
+          <t>uvm_scoreboard + SVA</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>risc_dec_00</t>
+          <t>risc_dec_03</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>All RV32I base instructions are legal and must execute correctly: LUI, AUIPC, JAL, JALR, BEQ, BNE, BLT, BGE, BLTU, BGEU, LB, LH, LW, LBU, LHU, SB, SH, SW, ADDI, SLTI, SLTIU, XORI, ORI, ANDI, SLLI, SRLI, SRAI, ADD, SUB, SLL, SLT, SLTU, XOR, SRL, SRA, OR, AND. (FENCE/FENCE.I/ECALL/EBREAK are part of the base but are excluded from stimulus per guideline Team4 Q2.)</t>
+          <t>Register operands equal to x0 keep legality: e.g. ADD x0,rs1,rs2, loads with rd=x0, JAL x0 (no link) are legal and produce the standard no-write/no-link behavior (see risc_rf_00); encodings that are undefined remain illegal even with x0 fields.</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>check every retired RV32I instruction against the golden model: rd value, memory effects, and next-PC</t>
+          <t>check via golden compare that x0-destination instructions retire with x0 unchanged and all other effects (e.g. JAL x0 still jumps) as per the ISA</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>sb_rv32i_result_match</t>
+          <t>sb_x0_zero, sb_pc_flow_match</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>sb (rvfi_pas_mon vs ref_model)</t>
+          <t>uvm_scoreboard</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>risc_dec_01</t>
+          <t>risc_alu_00</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>All 8 RV32M instructions are legal and must execute correctly: MUL, MULH, MULHSU, MULHU, DIV, DIVU, REM, REMU.</t>
+          <t>Integer computational instructions (ADD/SUB/AND/OR/XOR/SLL/SRL/SRA/SLT/SLTU + I-forms, LUI, AUIPC) produce their result in 1 cycle; the EX-&gt;ID forwarding path gives a 0-cycle penalty for a back-to-back dependent ALU instruction; SLT/SLTU distinguish signed vs unsigned compare and SLTIU compares rs1 unsigned against the sign-extended immediate (per the RISC-V spec).</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>check every retired RV32M instruction against the golden model (rd value and timing class)</t>
+          <t>check results via golden compare incl. forwarding chains (consumer equals producer value at distance 1,2,3)</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>sb_rv32m_result_match</t>
+          <t>sb_rv32i_result_match</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>sb</t>
+          <t>uvm_scoreboard</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>risc_dec_02</t>
+          <t>risc_alu_01</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>Illegal instruction detection (verified against cv32e40p_decoder.sv illegal_insn conditions): any encoding undefined for the configured parameter set raises an illegal instruction exception, including:
-(a) undefined major opcodes;
-(b) legal major opcode with undefined funct3/funct7 combination;
-(c) reserved shift encodings: OP-IMM/OP with funct3=001/101 and imm[11:5] (funct7) other than 0000000 or 0100000;
-(d) F / D / A major opcodes (FPU=0, atomics removed); (e) SYSTEM/CSR instructions accessing unimplemented CSR addresses; (f) CORE-V custom opcode spaces (incl. 0x0B, 0x2B, 0x5B, 0x7B) while COREV_PULP=0 / COREV_CLUSTER=0.</t>
+          <t>Shifts use a single-cycle barrel shifter; the shift amount shamt is operand_b[4:0] (register form) or imm[4:0]; SRA/SRAI replicate the sign bit; SLL/SRL shift in zeros. shamt=0 leaves the operand unchanged.</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>check that each injected illegal encoding is detected: the instruction retires to trap (no rd write, no memory request produced by it) and fetch redirects to mtvec base</t>
+          <t>check shift results via golden compare for every shamt corner and sign combination</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>sb_illegal_trap, exc_trap_base_prop</t>
+          <t>sb_shift_result_match</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t>sb + SVA</t>
+          <t>uvm_scoreboard</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>risc_dec_03</t>
+          <t>risc_alu_02</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>Trap state update on illegal instruction: mepc &lt;- PC of the offending instruction, mcause &lt;- 2 (illegal instruction), mstatus.MPIE/MIE update; PC &lt;- mtvec base. CSR content verification itself is out of scope; the architecturally visible effect (fetch redirect, no side effects) is checked, and mepc/mcause are probed only optionally.</t>
+          <t>LUI writes imm[31:12]&lt;&lt;12; AUIPC writes PC + (imm&lt;&lt;12) - the result depends on the current PC (position-dependent behavior).</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>check (design-visible part) redirect to mtvec base + zero architectural side effects of the trapped instruction. OPTIONAL (hierarchical): mepc == PC(illegal), mcause == 2</t>
+          <t>check AUIPC results across different PC regions (low/high boot locations, right after jumps)</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>sb_trap_redirect, sb_csr_sideband_opt</t>
+          <t>sb_upper_result_match</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t>sb; optional bind/hierarchical sample - CSR verification excluded per guideline Team3</t>
+          <t>uvm_scoreboard</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>risc_dec_04</t>
+          <t>risc_m_00</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>Register operands equal to x0 keep legality: e.g. ADD x0,rs1,rs2, loads with rd=x0, JAL x0 (no link) are legal and produce the standard no-write/no-link behavior (see risc_rf_00); encodings that are undefined remain illegal even with x0 fields.</t>
+          <t>MUL executes in 1 cycle (32x32 single-cycle multiplier, lower 32 bits of the product).</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>check via golden compare that x0-destination instructions retire with x0 unchanged and all other effects (e.g. JAL x0 jumps) as per ISA</t>
+          <t>check MUL result == lower-32 product via golden compare</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>sb_x0_zero, sb_pc_flow_match</t>
+          <t>sb_mul_result_match</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t>sb</t>
+          <t>uvm_scoreboard</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>risc_alu_00</t>
+          <t>risc_m_01</t>
         </is>
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>Integer computational instructions (ADD/SUB/AND/OR/XOR/SLL/SRL/SRA/SLT/SLTU + I-forms, LUI, AUIPC) produce their result in 1 cycle; the EX-&gt;ID forwarding path provides a 0-cycle penalty for a back-to-back dependent ALU instruction; SLT/SLTU distinguish signed vs unsigned compare and SLTIU compares rs1 unsigned against the sign-extended immediate (per RISC-V spec).</t>
+          <t>MULH/MULHSU/MULHU take 5 cycles (multicycle FSM STEP0-&gt;STEP1-&gt;STEP2-&gt;FINISH in rtl cv32e40p_mult.sv) and stall EX meanwhile; they return the upper 32 bits for signed x signed, signed x unsigned, unsigned x unsigned operands respectively.</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>check results via golden compare incl. forwarding chains (consumer equals producer value at distance 1,2,3)</t>
+          <t>check upper-half products for all three sign modes via golden compare; check no other write-back occurs during the stall window</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>sb_rv32i_result_match</t>
+          <t>sb_mulh_result_match, sb_no_spurious_wb</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t>sb</t>
+          <t>uvm_scoreboard (+ rvfi_monitor: single write per retire)</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>risc_alu_01</t>
+          <t>risc_m_02</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>Shifts use a single-cycle barrel shifter; shift amount shamt is operand_b[4:0] (reg form) or imm[4:0]; SRA/SRAI replicate the sign bit; SLL/SRL shift in zeros. shamt=0 leaves the operand unchanged.</t>
+          <t>DIV/DIVU/REM/REMU are iterative with early termination: latency is 3..35 cycles depending on the number of leading zeros of operand b (the divisor); minimum 3 cycles when the divisor has no leading zeros (e.g. 0x80000000), maximum 35 when the divisor is 0; EX stalls meanwhile.</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>check shift results via golden compare for every shamt corner and sign combination</t>
+          <t>check div/rem results via golden compare AND measured retire-latency within 3..35 cycles at zero wait states</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>sb_shift_result_match</t>
+          <t>sb_div_result_match, sb_div_latency_range</t>
         </is>
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t>sb</t>
+          <t>uvm_scoreboard (latency measured between issue and retire at zero wait states)</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>risc_alu_02</t>
+          <t>risc_m_03</t>
         </is>
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>LUI writes imm[31:12]&lt;&lt;12; AUIPC writes PC + (imm&lt;&lt;12) - the value depends on the current PC (position-dependent behavior).</t>
+          <t>Special division results per the RISC-V spec: divide-by-zero -&gt; quotient = -1 (all ones) for DIV/DIVU; remainder = dividend for REM/REMU. Signed overflow (DIV -2^31 / -1) -&gt; quotient = -2^31, REM -2^31 / -1 -&gt; 0. The REM sign follows the dividend; REMU is unsigned.</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>check AUIPC results across different PC regions (low/high boot locations, after jumps)</t>
+          <t>check the exact special-case values via golden compare (directed vectors)</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>sb_upper_result_match</t>
+          <t>sb_div_corner_results</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
         <is>
-          <t>sb</t>
+          <t>uvm_scoreboard</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>risc_m_00</t>
+          <t>risc_m_04</t>
         </is>
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>MUL executes in 1 cycle (32x32 single-cycle multiplier, lower 32 bits of the product).</t>
+          <t>A multicycle instruction (MULH/DIV/REM) that is older than a taken branch always completes and writes back normally, even when the flush of the younger path lands in the same window - only IF/ID (the younger stages) are flushed.</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>check MUL result == lower-32 product via golden compare</t>
+          <t>check the multicycle result is written back and the branch-target path retires correctly (scenario test)</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>sb_mul_result_match</t>
+          <t>sb_multicycle_plus_branch</t>
         </is>
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t>sb</t>
+          <t>uvm_scoreboard</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>risc_m_01</t>
+          <t>risc_haz_00</t>
         </is>
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>MULH/MULHSU/MULHU take 5 cycles (multicycle FSM STEP0-&gt;STEP1-&gt;STEP2-&gt;FINISH in rtl cv32e40p_mult.sv) and stall EX meanwhile; they return the upper 32 bits for signed x signed, signed x unsigned, unsigned x unsigned operands respectively.</t>
+          <t>RAW forwarding: ALU/MUL/DIV results in EX are forwarded to ID-stage operands (ports a and b), giving a 0-cycle penalty for back-to-back dependent instructions; the consumer reads correct producer values at distance 1, 2, 3.</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>check upper-half products for all three sign modes via golden compare; check no other write-back occurs during the stall window</t>
+          <t>check consumer results via golden compare across dependency distances and both operand slots</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>sb_mulh_result_match, sb_no_spurious_wb</t>
+          <t>sb_rv32i_result_match</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t>sb (+ rvfi single-write per retire)</t>
+          <t>uvm_scoreboard (guaranteed through dense dependent streams)</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
         <is>
-          <t>risc_m_02</t>
+          <t>risc_haz_01</t>
         </is>
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>DIV/DIVU/REM/REMU are iterative with early termination: latency is 3..35 cycles depending on the number of leading zeros of operand b (divisor); minimum 3 cycles when the divisor has no leading zeros (e.g. 0x80000000), maximum 35 when the divisor is 0; EX stalls meanwhile.</t>
+          <t>Load-use hazard: an instruction consuming a register written by the immediately preceding load is stalled exactly 1 cycle (controller load_stall + deassert_we in rtl cv32e40p_controller.sv); no wrong value is read and no spurious write occurs during the stall.</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>check div/rem results via golden compare AND measured retire-latency within 3..35 cycles at zero wait states</t>
+          <t>check the consumer receives the load data (golden compare) and the retire spacing shows the single stall cycle at zero wait states</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>sb_div_result_match, sb_div_latency_range</t>
+          <t>sb_load_use_correct, sb_load_use_1cycle</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t>sb (latency measured between issue and retire at zero-wait)</t>
+          <t>uvm_scoreboard</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
         <is>
-          <t>risc_m_03</t>
+          <t>risc_haz_02</t>
         </is>
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>Special division results per RISC-V spec: Divide-by-zero -&gt; quotient = -1 (all ones) for DIV/DIVU; remainder = dividend for REM/REMU. Signed overflow (DIV -2^31 / -1) -&gt; quotient = -2^31, REM -2^31 / -1 -&gt; 0. REM sign follows the dividend; REMU is unsigned.</t>
+          <t>JALR data hazard: a JALR whose rs1 is produced by the immediately preceding instruction is stalled 1 cycle (jr_stall) before computing its target; the target must be (rs1+imm) &amp; ~1.</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>check the exact special-case values via golden compare (directed vectors)</t>
+          <t>check JALR target correctness when rs1 comes from an ALU result and from a load result, via golden compare of the PC stream</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>sb_div_corner_results</t>
+          <t>sb_jalr_target_match</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t>sb</t>
+          <t>uvm_scoreboard</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
         <is>
-          <t>risc_m_04</t>
+          <t>risc_haz_03</t>
         </is>
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>A multicycle instruction (MULH/DIV/REM) that is older than a taken branch always completes and writes back normally even if the flush of younger instructions happens in the same window (answer to open guideline question Team4 Q4, resolved from databook pipeline chapter and rtl: only IF/ID - i.e. younger instructions - are flushed).</t>
+          <t>WAW write-port arbitration: a load in WB and a younger ALU/MUL/DIV instruction in EX may write the same rd in the same cycle; the register file resolves it with port-b (EX) priority, i.e. the architecturally younger instruction wins (verified in rtl cv32e40p_register_file_ff.sv: the we_b write is checked before we_a).</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>check the multicycle result is written back and the branch target path retires correctly (scenario test)</t>
+          <t>check that after such a collision the final rd value equals the younger instruction's result (golden model final-state compare + targeted readback)</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>sb_multicycle_plus_branch</t>
+          <t>sb_waw_younger_wins</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t>sb</t>
+          <t>uvm_scoreboard</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
-          <t>risc_haz_00</t>
+          <t>risc_haz_04</t>
         </is>
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>RAW forwarding: ALU/MUL/DIV results in EX are forwarded to ID-stage operands (ports a and b), giving 0-cycle penalty for back-to-back dependent instructions; the consumer reads correct producer values at distance 1, 2, 3.</t>
+          <t>Control-flush cleanliness: instructions younger than a taken branch / jump / trap never produce architectural side effects (no register write, no memory request).</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>check consumer results via golden compare across dependency distances and both operand slots</t>
+          <t>check per retire stream + data-bus log: nothing from the flushed path appears (companion to risc_if_06 and risc_lsu_08)</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>sb_rv32i_result_match</t>
+          <t>sb_flush_clean, sb_lsu_trans_stream_match</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t>sb (guaranteed through dense dependent streams)</t>
+          <t>uvm_scoreboard</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t>risc_haz_01</t>
+          <t>risc_rf_00</t>
         </is>
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>Load-use hazard: an instruction consuming a register written by the immediately preceding load is stalled exactly 1 cycle (controller load_stall + deassert_we in rtl cv32e40p_controller.sv); no wrong value is read and no spurious write occurs during the stall.</t>
+          <t>x0 is hardwired to zero: reads always return 0 and writes to x0 are ignored (x0 has no flip-flops), even when a load targets x0.</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>check consumer receives load data (golden compare) and retire spacing shows the single stall cycle at zero wait states</t>
+          <t>check x0==0 after every retired instruction (monitor side) and that x0-source operands are read as 0 (covered by the golden compare)</t>
         </is>
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>sb_load_use_correct, sb_load_use_1cycle</t>
+          <t>sb_x0_zero</t>
         </is>
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t>sb</t>
+          <t>uvm_scoreboard / optional hierarchical SVA on RF mem[0]</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
         <is>
-          <t>risc_haz_02</t>
+          <t>risc_rf_01</t>
         </is>
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>JALR data hazard: a JALR whose rs1 is produced by the immediately preceding instruction is stalled 1 cycle (jr_stall) before computing its target; the target must be (rs1+imm) &amp; ~1.</t>
+          <t>All 31 general-purpose registers x1..x31 are implemented (the FF register file resets to 0 at rst_ni==0) with 3 read ports and 2 write ports; reads happen in ID, writes from EX and WB.</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>check JALR target correctness when rs1 comes from ALU result and from load result, via golden compare of the PC stream</t>
+          <t>check initial reads of unwritten registers return 0 (first test only, implementation-specific), afterwards golden compare</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>sb_jalr_target_match</t>
+          <t>sb_rf_reset_zero_opt</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t>sb</t>
+          <t>uvm_scoreboard; optional, documented as implementation-specific</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
         <is>
-          <t>risc_haz_03</t>
+          <t>risc_rst_00</t>
         </is>
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>WAW write-port arbitration: a load in WB and a younger ALU/MUL/DIV instruction in EX may write the same rd in the same cycle; the register file resolves it with port-b (EX) priority, i.e. the architecturally younger instruction wins (open guideline question Team4 Q6, answered directly from rtl cv32e40p_register_file_ff.sv: we_b checked before we_a).</t>
+          <t>Reset re-assertion during an outstanding instruction-fetch transaction: core and TB slave both drop the transaction; after re-enabling, the core re-boots from boot_addr_i with a clean pipeline; no stale rvalid may be consumed after reset.</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>check that after such a collision the final rd value equals the younger instruction's result (golden model final-state compare + targeted readback)</t>
+          <t>check post-reset re-boot: first fetch == boot_addr_i, the scoreboard re-syncs, zero mismatches afterwards</t>
         </is>
       </c>
       <c r="D43" s="5" t="inlineStr">
         <is>
-          <t>sb_waw_younger_wins</t>
+          <t>sb_reset_resync</t>
         </is>
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t>sb</t>
+          <t>uvm_scoreboard</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="5" t="inlineStr">
         <is>
-          <t>risc_haz_04</t>
+          <t>risc_rst_01</t>
         </is>
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>Control-flush cleanliness: instructions younger than a taken branch / jump / trap never produce architectural side effects (no register write, no memory request).</t>
+          <t>Reset re-assertion during outstanding data transactions (load/store granted but rvalid pending, incl. mid misaligned pair).</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>check per retire stream + data-bus log: nothing from the flushed path appears (companion to risc_if_06 and risc_lsu_08)</t>
+          <t>check post-reset re-boot and no corruption of the dmem image (stores before reset kept, partial pair never completed)</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>sb_flush_clean, sb_lsu_trans_stream_match</t>
+          <t>sb_reset_resync, sb_store_mem_match</t>
         </is>
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t>sb</t>
+          <t>uvm_scoreboard</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
         <is>
-          <t>risc_rf_00</t>
+          <t>risc_rst_02</t>
         </is>
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>x0 is hardwired to zero: reads always return 0 and writes to x0 are ignored (x0 has no flip-flops), even when a load targets x0.</t>
+          <t>Reset re-assertion during a multicycle DIV/REM or MULH execution, and during a branch-flush window.</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>check x0==0 after every retired instruction (monitor) and that x0-source operands are read as 0 (golden compare covers this)</t>
+          <t>check post-reset re-boot; no write-back from the killed multicycle instruction appears after reset</t>
         </is>
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>sb_x0_zero</t>
+          <t>sb_reset_resync, sb_no_spurious_wb</t>
         </is>
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t>sb/SVA on RF mem[0] optionally hierarchical</t>
+          <t>uvm_scoreboard</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="5" t="inlineStr">
         <is>
-          <t>risc_rf_01</t>
+          <t>risc_env_01</t>
         </is>
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>All 31 general-purpose registers x1..x31 are implemented (FF register file resets to 0 at rst_ni==0) with 3 read ports and 2 write ports; reads happen in ID, writes from EX and WB.</t>
+          <t>OBI slave response features: per-transaction gnt delay (0..K), rvalid delay (1..L); operating modes: zero-wait, random, long-stall bursts, gnt-always-high; both buses configurable independently.</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>check initial reads of unwritten registers return 0 (first test only, implementation-specific), afterwards golden compare</t>
+          <t>check slave protocol self-guards (never two rvalid for one grant; never rvalid with an empty outstanding queue; rdata stable at the rvalid cycle)</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>sb_rf_reset_zero_opt</t>
+          <t>env_slave_protocol_prop</t>
         </is>
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t>sb; optional, documented as implementation-specific</t>
+          <t>Assertions inside if_agent / lsu_agent drivers</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t>risc_rst_00</t>
+          <t>risc_env_02</t>
         </is>
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>Reset re-assertion during an outstanding instruction-fetch transaction: core and TB slave both drop the transaction; after re-enabling, the core re-boots from boot_addr_i with a clean pipeline; no stale rvalid may be consumed after reset.</t>
+          <t>Test teardown: at end of test all outstanding responses are delivered (memory drains), the retire stream is checked complete against expectations, and the final GPR + memory state is compared; a global watchdog timeout catches any hung core.</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>check post-reset re-boot: first fetch == boot_addr_i, scoreboard re-syncs, zero mismatches afterwards</t>
+          <t>check end-of-test flush: outstanding==0 on both buses, final register file contents == golden, final dmem == golden, no test timeout</t>
         </is>
       </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>sb_reset_resync</t>
+          <t>sb_final_state_match, env_teardown_check</t>
         </is>
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t>sb</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="5" t="inlineStr">
-        <is>
-          <t>risc_rst_01</t>
-        </is>
-      </c>
-      <c r="B48" s="5" t="inlineStr">
-        <is>
-          <t>Reset re-assertion during outstanding data transactions (load/store granted but rvalid pending, incl. mid misaligned pair).</t>
-        </is>
-      </c>
-      <c r="C48" s="5" t="inlineStr">
-        <is>
-          <t>check post-reset re-boot and no corruption of the dmem image (stores before reset kept, partial pair never completed)</t>
-        </is>
-      </c>
-      <c r="D48" s="5" t="inlineStr">
-        <is>
-          <t>sb_reset_resync, sb_store_mem_match</t>
-        </is>
-      </c>
-      <c r="E48" s="5" t="inlineStr">
-        <is>
-          <t>sb</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="5" t="inlineStr">
-        <is>
-          <t>risc_rst_02</t>
-        </is>
-      </c>
-      <c r="B49" s="5" t="inlineStr">
-        <is>
-          <t>Reset re-assertion during a multicycle DIV/REM or MULH execution, and during a branch-flush window.</t>
-        </is>
-      </c>
-      <c r="C49" s="5" t="inlineStr">
-        <is>
-          <t>check post-reset re-boot; no write-back from the killed multicycle instruction appears after reset</t>
-        </is>
-      </c>
-      <c r="D49" s="5" t="inlineStr">
-        <is>
-          <t>sb_reset_resync, sb_no_spurious_wb</t>
-        </is>
-      </c>
-      <c r="E49" s="5" t="inlineStr">
-        <is>
-          <t>sb</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="5" t="inlineStr">
-        <is>
-          <t>risc_env_01</t>
-        </is>
-      </c>
-      <c r="B50" s="5" t="inlineStr">
-        <is>
-          <t>OBI slave response generation features: per-transaction gnt delay (0..K), rvalid delay (1..L), operating modes: zero-wait, random, long-stall bursts, gnt-always-high; both buses independently configurable.</t>
-        </is>
-      </c>
-      <c r="C50" s="5" t="inlineStr">
-        <is>
-          <t>check slave protocol self-guards (never two rvalid for one grant; never rvalid with empty outstanding queue; rdata stable at rvalid)</t>
-        </is>
-      </c>
-      <c r="D50" s="5" t="inlineStr">
-        <is>
-          <t>env_slave_protocol_prop</t>
-        </is>
-      </c>
-      <c r="E50" s="5" t="inlineStr">
-        <is>
-          <t>env assertions</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="5" t="inlineStr">
-        <is>
-          <t>risc_env_02</t>
-        </is>
-      </c>
-      <c r="B51" s="5" t="inlineStr">
-        <is>
-          <t>Test teardown: at end of test all outstanding responses are delivered (memory drains), the retire stream is empty-checked against expectations, and the final GPR + memory state is compared; a global watchdog timeout catches any hung core.</t>
-        </is>
-      </c>
-      <c r="C51" s="5" t="inlineStr">
-        <is>
-          <t>check end-of-test flush: outstanding==0 on both buses, final regfile contents == golden, final dmem == golden, no test timeout</t>
-        </is>
-      </c>
-      <c r="D51" s="5" t="inlineStr">
-        <is>
-          <t>sb_final_state_match, env_teardown_check</t>
-        </is>
-      </c>
-      <c r="E51" s="5" t="inlineStr">
-        <is>
-          <t>sb</t>
+          <t>uvm_scoreboard</t>
         </is>
       </c>
     </row>
@@ -4183,7 +4000,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>fetch_enable_i: the first instruction fetch after reset de-assertion must not happen while fetch_enable_i==0; after fetch_enable_i has been 1 for at least one cycle (out of reset) fetching starts permanently, and the value of fetch_enable_i is ignored until the next reset. boot_addr_i/mtvec_addr_i/dm_*_addr_i/hart_id_i must stay stable once enabled.</t>
+          <t>fetch_enable_i: the first instruction fetch after reset de-assertion must not happen while fetch_enable_i==0; after fetch_enable_i has been 1 for at least one cycle (out of reset) fetching starts permanently, and the value of fetch_enable_i is ignored until the next reset. boot_addr_i / mtvec_addr_i / dm_*_addr_i / hart_id_i must stay stable once the core is enabled.</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
@@ -4232,7 +4049,7 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Cover the case gnt_i==1 while req_o==0 on IF channel (phi window)</t>
+          <t>Cover the case gnt_i==1 while req_o==0 on the IF channel</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
@@ -4293,7 +4110,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Flush on taken jump (JAL/JALR are resolved in ID stage): the prefetch buffer and IF stage are flushed; the new PC request appears on the instruction-side memory interface in the same cycle the jump is in ID; with zero wait states the jump costs 2 cycles.</t>
+          <t>Flush on taken jump (JAL/JALR are resolved in the ID stage): the prefetch buffer and IF stage are flushed; the new PC request appears on the instruction-side memory interface in the same cycle the jump is in ID; with zero wait states the jump costs 2 cycles.</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
@@ -4315,12 +4132,12 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Flush on taken branch (resolved in EX stage): IF stage and ID stage are flushed; fetch restarts at the branch target; with zero wait states a taken branch costs 3 cycles; a not-taken branch costs 1 cycle (no stall).</t>
+          <t>Flush on taken branch (resolved in the EX stage): the IF stage and ID stage are flushed; fetch restarts at the branch target; with zero wait states a taken branch costs 3 cycles; a not-taken branch costs 1 cycle (no stall).</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Cover each branch x taken/not-taken x direction x operand-relation; cover taken branch while the target fetch encounters wait states</t>
+          <t>Cover each branch x taken/not-taken x direction x operand-relation; cover a taken branch while the target fetch encounters wait states</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
@@ -4359,7 +4176,7 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Data OBI handshake: data_req_o is raised for load/store and must stay high until data_gnt_i is sampled high; data_addr_o, data_we_o, data_be_o, data_wdata_o are send together with the request and must stay stable while req==1 &amp;&amp; gnt==0.</t>
+          <t>Data OBI handshake: data_req_o is raised for load/store and must stay high until data_gnt_i is sampled high; data_addr_o, data_we_o, data_be_o, data_wdata_o are sent together with the request and must stay stable while req==1 &amp;&amp; gnt==0.</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
@@ -4386,7 +4203,7 @@
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Cover data outstanding-depth bins 1 and 2; cover LSU rvalid latency bins 1, 2, 3-7, &gt;7; cover stall during second phase of a misaligned pair</t>
+          <t>Cover data outstanding-depth bins 1 and 2; cover LSU rvalid latency bins 1, 2, 3-7, &gt;7; cover stall during the second phase of a misaligned pair</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
@@ -4429,7 +4246,7 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>Misaligned handling: the LSU never raises address-misaligned exceptions. A word load/store at addr[1:0]!=00, or a halfword at addr[1:0]==11, is performed as TWO bus transactions; the transfer for the lowest address is issued first, followed by (aligned base+4) with the complementary byte-enables; the core spends 2 cycles each in EX and WB per part and merges the response data. All other offsets need a single transaction.</t>
+          <t>Misaligned handling: the LSU never raises address-misaligned exceptions. A word load/store at addr[1:0]!=00, or a halfword at addr[1:0]==11, is performed as TWO bus transactions; the transfer for the lowest address is issued first, followed by (aligned base+4) with the complementary byte-enables; the memory transfers for the two parts are merged by the core into one load/store view. All other offsets need a single transaction.</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
@@ -4473,7 +4290,7 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>Load data alignment and extension: LB/LH sign-extend the addressed byte/halfword; LBU/LHU zero-extend; LW returns the full word; for misaligned accesses the two response words are assembled (first-response low bytes kept in rdata_q, combined with second response) according to the address offset.</t>
+          <t>Load data alignment and extension: LB/LH sign-extend the addressed byte/halfword; LBU/LHU zero-extend; LW returns the full word; for misaligned accesses the two response words are assembled (first-response low bytes kept in rdata_q, combined with the second response) according to the address offset.</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
@@ -4495,7 +4312,7 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>Memory consistency: in-order data responses + single hart imply a load must observe the value of the most recent previously-issued store to the same byte address; the TB memory model commits a store at its rvalid and never reorders.</t>
+          <t>Memory consistency: in-order data responses and a single hart imply a load must observe the value of the most recent previously-issued store to the same byte address; the TB memory model commits a store at its rvalid and never reorders.</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
@@ -4539,7 +4356,7 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>All RV32I base instructions are legal and must execute correctly: LUI, AUIPC, JAL, JALR, BEQ, BNE, BLT, BGE, BLTU, BGEU, LB, LH, LW, LBU, LHU, SB, SH, SW, ADDI, SLTI, SLTIU, XORI, ORI, ANDI, SLLI, SRLI, SRAI, ADD, SUB, SLL, SLT, SLTU, XOR, SRL, SRA, OR, AND. (FENCE/FENCE.I/ECALL/EBREAK are part of the base but are excluded from stimulus per guideline Team4 Q2.)</t>
+          <t>All RV32I base instructions are legal and must execute correctly: LUI, AUIPC, JAL, JALR, BEQ, BNE, BLT, BGE, BLTU, BGEU, LB, LH, LW, LBU, LHU, SB, SH, SW, ADDI, SLTI, SLTIU, XORI, ORI, ANDI, SLLI, SRLI, SRAI, ADD, SUB, SLL, SLT, SLTU, XOR, SRL, SRA, OR, AND. (FENCE / FENCE.I / ECALL / EBREAK are part of the base ISA but are omitted from the generated stimulus.)</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
@@ -4583,16 +4400,15 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>Illegal instruction detection (verified against cv32e40p_decoder.sv illegal_insn conditions): any encoding undefined for the configured parameter set raises an illegal instruction exception, including:
+          <t>Illegal instruction detection within the RV32I/M opcode space (verified against cv32e40p_decoder.sv illegal_insn conditions): any undefined encoding raises an illegal instruction exception, including:
 (a) undefined major opcodes;
-(b) legal major opcode with undefined funct3/funct7 combination;
-(c) reserved shift encodings: OP-IMM/OP with funct3=001/101 and imm[11:5] (funct7) other than 0000000 or 0100000;
-(d) F / D / A major opcodes (FPU=0, atomics removed); (e) SYSTEM/CSR instructions accessing unimplemented CSR addresses; (f) CORE-V custom opcode spaces (incl. 0x0B, 0x2B, 0x5B, 0x7B) while COREV_PULP=0 / COREV_CLUSTER=0.</t>
+(b) a legal major opcode with an undefined funct3/funct7 combination;
+(c) reserved shift encodings: OP-IMM/OP with funct3=001/101 and imm[11:5] (funct7) other than 0000000 or 0100000.</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>Cover each illegal category (a)-(f) at least once; cover illegal back-to-back and illegal during OBI wait-state windows</t>
+          <t>Cover each illegal category (a)-(c) at least once; cover illegal back-to-back and illegal during OBI wait-state windows</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
@@ -4604,7 +4420,7 @@
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>risc_dec_04</t>
+          <t>risc_dec_03</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
@@ -4631,7 +4447,7 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>Integer computational instructions (ADD/SUB/AND/OR/XOR/SLL/SRL/SRA/SLT/SLTU + I-forms, LUI, AUIPC) produce their result in 1 cycle; the EX-&gt;ID forwarding path provides a 0-cycle penalty for a back-to-back dependent ALU instruction; SLT/SLTU distinguish signed vs unsigned compare and SLTIU compares rs1 unsigned against the sign-extended immediate (per RISC-V spec).</t>
+          <t>Integer computational instructions (ADD/SUB/AND/OR/XOR/SLL/SRL/SRA/SLT/SLTU + I-forms, LUI, AUIPC) produce their result in 1 cycle; the EX-&gt;ID forwarding path gives a 0-cycle penalty for a back-to-back dependent ALU instruction; SLT/SLTU distinguish signed vs unsigned compare and SLTIU compares rs1 unsigned against the sign-extended immediate (per the RISC-V spec).</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
@@ -4653,7 +4469,7 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>Shifts use a single-cycle barrel shifter; shift amount shamt is operand_b[4:0] (reg form) or imm[4:0]; SRA/SRAI replicate the sign bit; SLL/SRL shift in zeros. shamt=0 leaves the operand unchanged.</t>
+          <t>Shifts use a single-cycle barrel shifter; the shift amount shamt is operand_b[4:0] (register form) or imm[4:0]; SRA/SRAI replicate the sign bit; SLL/SRL shift in zeros. shamt=0 leaves the operand unchanged.</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
@@ -4675,12 +4491,12 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>LUI writes imm[31:12]&lt;&lt;12; AUIPC writes PC + (imm&lt;&lt;12) - the value depends on the current PC (position-dependent behavior).</t>
+          <t>LUI writes imm[31:12]&lt;&lt;12; AUIPC writes PC + (imm&lt;&lt;12) - the result depends on the current PC (position-dependent behavior).</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>Cover AUIPC at diverse PC values (cross with branch target regions)</t>
+          <t>Cover AUIPC at diverse PC values (cross with branch-target regions)</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
@@ -4741,7 +4557,7 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>DIV/DIVU/REM/REMU are iterative with early termination: latency is 3..35 cycles depending on the number of leading zeros of operand b (divisor); minimum 3 cycles when the divisor has no leading zeros (e.g. 0x80000000), maximum 35 when the divisor is 0; EX stalls meanwhile.</t>
+          <t>DIV/DIVU/REM/REMU are iterative with early termination: latency is 3..35 cycles depending on the number of leading zeros of operand b (the divisor); minimum 3 cycles when the divisor has no leading zeros (e.g. 0x80000000), maximum 35 when the divisor is 0; EX stalls meanwhile.</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
@@ -4763,7 +4579,7 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>Special division results per RISC-V spec: Divide-by-zero -&gt; quotient = -1 (all ones) for DIV/DIVU; remainder = dividend for REM/REMU. Signed overflow (DIV -2^31 / -1) -&gt; quotient = -2^31, REM -2^31 / -1 -&gt; 0. REM sign follows the dividend; REMU is unsigned.</t>
+          <t>Special division results per the RISC-V spec: divide-by-zero -&gt; quotient = -1 (all ones) for DIV/DIVU; remainder = dividend for REM/REMU. Signed overflow (DIV -2^31 / -1) -&gt; quotient = -2^31, REM -2^31 / -1 -&gt; 0. The REM sign follows the dividend; REMU is unsigned.</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
@@ -4785,7 +4601,7 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>A multicycle instruction (MULH/DIV/REM) that is older than a taken branch always completes and writes back normally even if the flush of younger instructions happens in the same window (answer to open guideline question Team4 Q4, resolved from databook pipeline chapter and rtl: only IF/ID - i.e. younger instructions - are flushed).</t>
+          <t>A multicycle instruction (MULH/DIV/REM) that is older than a taken branch always completes and writes back normally, even when the flush of the younger path lands in the same window - only IF/ID (the younger stages) are flushed.</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
@@ -4807,7 +4623,7 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>RAW forwarding: ALU/MUL/DIV results in EX are forwarded to ID-stage operands (ports a and b), giving 0-cycle penalty for back-to-back dependent instructions; the consumer reads correct producer values at distance 1, 2, 3.</t>
+          <t>RAW forwarding: ALU/MUL/DIV results in EX are forwarded to ID-stage operands (ports a and b), giving a 0-cycle penalty for back-to-back dependent instructions; the consumer reads correct producer values at distance 1, 2, 3.</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
@@ -4873,12 +4689,12 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>WAW write-port arbitration: a load in WB and a younger ALU/MUL/DIV instruction in EX may write the same rd in the same cycle; the register file resolves it with port-b (EX) priority, i.e. the architecturally younger instruction wins (open guideline question Team4 Q6, answered directly from rtl cv32e40p_register_file_ff.sv: we_b checked before we_a).</t>
+          <t>WAW write-port arbitration: a load in WB and a younger ALU/MUL/DIV instruction in EX may write the same rd in the same cycle; the register file resolves it with port-b (EX) priority, i.e. the architecturally younger instruction wins (verified in rtl cv32e40p_register_file_ff.sv: the we_b write is checked before we_a).</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>Cover collision window positions (load WB overlapping EX write)</t>
+          <t>Cover collision window positions (load WB overlapping the EX write)</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
@@ -4895,7 +4711,7 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>All 31 general-purpose registers x1..x31 are implemented (FF register file resets to 0 at rst_ni==0) with 3 read ports and 2 write ports; reads happen in ID, writes from EX and WB.</t>
+          <t>All 31 general-purpose registers x1..x31 are implemented (the FF register file resets to 0 at rst_ni==0) with 3 read ports and 2 write ports; reads happen in ID, writes from EX and WB.</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
@@ -4983,7 +4799,7 @@
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>OBI slave response generation features: per-transaction gnt delay (0..K), rvalid delay (1..L), operating modes: zero-wait, random, long-stall bursts, gnt-always-high; both buses independently configurable.</t>
+          <t>OBI slave response features: per-transaction gnt delay (0..K), rvalid delay (1..L); operating modes: zero-wait, random, long-stall bursts, gnt-always-high; both buses configurable independently.</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
@@ -5058,7 +4874,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>Apply reset (random delay/hold), program boot_addr_i/mtvec_addr_i at corner values, toggle fetch_enable at 0/1/N cycles; check boot flow and output inactivity; repeat with 2nd reset mid-idle. Multiple seeds.</t>
+          <t>Apply reset (random delay/hold), program boot_addr_i/mtvec_addr_i at corner values, toggle fetch_enable at 0/1/N cycles; check boot flow and output inactivity; repeat with a 2nd reset mid-idle. Multiple seeds.</t>
         </is>
       </c>
     </row>
@@ -5075,7 +4891,7 @@
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>Sweep fetch_enable delays incl. &gt;8 cycles; verify no fetch before enable and permanent activity after (pure behavioral test).</t>
+          <t>Sweep fetch_enable delays incl. &gt;8 cycles; verify no fetch before enable and permanent activity after.</t>
         </is>
       </c>
     </row>
@@ -5177,7 +4993,7 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>LB/LBU/LH/LHU loads where target byte/half MSB toggles 0/1 at every offset; verify sign vs zero extension. ~1000 instrs.</t>
+          <t>LB/LBU/LH/LHU loads where the target byte/half MSB toggles 0/1 at every offset; verify sign vs zero extension. ~1000 instrs.</t>
         </is>
       </c>
     </row>
@@ -5245,7 +5061,7 @@
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>JAL fwd/back with link x0/x1/x5; JALR with odd/even immediates (and ~1 rule), various base registers. ~1500 jumps.</t>
+          <t>JAL fwd/back with link x0/x1/x5; JALR with odd/even immediates (&amp; ~1 rule), various base registers. ~1500 jumps.</t>
         </is>
       </c>
     </row>
@@ -5330,7 +5146,7 @@
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>Inject illegal encodings of every category (a)-(f) at random positions; check trap redirect, no side effects, resume at handler. ~1000 injections.</t>
+          <t>Inject illegal encodings of every category (a)-(c) at random positions; check trap redirect, no side effects, resume at handler. ~1000 injections.</t>
         </is>
       </c>
     </row>
@@ -5398,7 +5214,7 @@
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>LW rd followed by ALU/MUL/DIV writing same rd at 1..3 spacing; targeted readback of rd afterwards. ~1000 scenarios.</t>
+          <t>LW rd followed by ALU/MUL/DIV writing the same rd at 1..3 spacing (incl. misaligned-load producer); targeted readback of rd afterwards. ~1000 scenarios.</t>
         </is>
       </c>
     </row>
@@ -5449,7 +5265,7 @@
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>Long-stall bursts forced during mem-heavy windows to saturate 2-outstanding LSU and 2-outstanding prefetch; stall during misaligned 2nd beat targeted.</t>
+          <t>Long-stall bursts forced during mem-heavy windows to saturate 2-outstanding LSU and 2-outstanding prefetch; stall during the misaligned 2nd beat targeted.</t>
         </is>
       </c>
     </row>
@@ -5466,7 +5282,7 @@
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>gnt held high for long windows incl. while no request pending, on both IF and LSU channels.</t>
+          <t>gnt held high for long windows incl. while no request is pending, on both IF and LSU channels.</t>
         </is>
       </c>
     </row>
@@ -5500,7 +5316,7 @@
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>Fully random RV32IM program streams (weighted classes incl. illegals ratio ~2%) + random OBI delays both buses; main regression test. ~5000 instrs x 30 seeds.</t>
+          <t>Fully random RV32IM program streams (weighted classes incl. illegals ratio ~2%) + random OBI delays on both buses; main regression test. ~5000 instrs x 30 seeds.</t>
         </is>
       </c>
     </row>

</xml_diff>